<commit_message>
feat: add Zoom In management page with event handling and translations
- Implemented Zoom In page for managing events, including fetching, displaying, and deleting events.
- Added pagination and search functionality for event listings.
- Integrated user permissions for viewing, editing, and deleting events.
- Created translations for Zoom In management, including event types, activities, and allocations.
- Updated API error handling to improve user feedback on validation errors.
- Enhanced navigation with new Zoom In related items.
</commit_message>
<xml_diff>
--- a/backend/data/emplyoees.xlsx
+++ b/backend/data/emplyoees.xlsx
@@ -5,20 +5,21 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\sadekinislam\projects\Orange-Flow-Next-Js\backend\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\emil\projects\Orange-Flow-Next-Js\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5680A2A6-0A6A-4E7D-B077-ABBBAAD2FBFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D828ED5-2DF0-44DB-B4BB-491A0EF9ACAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AL$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AL$46</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="823" uniqueCount="359">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="867" uniqueCount="374">
   <si>
     <t>DMS_CODE</t>
   </si>
@@ -1116,6 +1117,51 @@
   </si>
   <si>
     <t>R364204</t>
+  </si>
+  <si>
+    <t>Inactive</t>
+  </si>
+  <si>
+    <t>Arif</t>
+  </si>
+  <si>
+    <t>Sanaullah</t>
+  </si>
+  <si>
+    <t>Kuliarchar Government High School</t>
+  </si>
+  <si>
+    <t>South Salua Dumrakanda, Kuliarchar, Kishoreganj.</t>
+  </si>
+  <si>
+    <t>Halima Begum</t>
+  </si>
+  <si>
+    <t>soliman</t>
+  </si>
+  <si>
+    <t>MER-RYZBRB0129</t>
+  </si>
+  <si>
+    <t>arif</t>
+  </si>
+  <si>
+    <t>R648020</t>
+  </si>
+  <si>
+    <t>Poshim Nandina</t>
+  </si>
+  <si>
+    <t>Md. Forid Mia</t>
+  </si>
+  <si>
+    <t>Bajitpur Government High School</t>
+  </si>
+  <si>
+    <t>West Nandina Aliabaad, Bajitpur, Kishoreganj.</t>
+  </si>
+  <si>
+    <t>Onufa</t>
   </si>
 </sst>
 </file>
@@ -1125,7 +1171,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]d/mmm/yy;@"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1153,6 +1199,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1174,7 +1227,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1226,6 +1279,9 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1566,7 +1622,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AL45"/>
+  <dimension ref="A1:AL50"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.5703125" style="5" bestFit="1" customWidth="1"/>
@@ -1590,7 +1646,7 @@
     <col min="19" max="19" width="16.7109375" style="7" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="15.140625" style="5" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="18.7109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="13.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="15.5703125" style="5" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="37.140625" style="5" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="39.7109375" style="5" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="13.85546875" style="5" bestFit="1" customWidth="1"/>
@@ -4167,7 +4223,7 @@
       <c r="D34" s="8" t="s">
         <v>168</v>
       </c>
-      <c r="E34" s="8" t="s">
+      <c r="E34" s="18" t="s">
         <v>169</v>
       </c>
       <c r="F34" s="8" t="s">
@@ -4255,7 +4311,7 @@
         <v>166</v>
       </c>
       <c r="AL34" s="8" t="s">
-        <v>74</v>
+        <v>359</v>
       </c>
     </row>
     <row r="35" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -4373,7 +4429,7 @@
       <c r="D36" s="8" t="s">
         <v>187</v>
       </c>
-      <c r="E36" s="8" t="s">
+      <c r="E36" s="18" t="s">
         <v>188</v>
       </c>
       <c r="F36" s="8" t="s">
@@ -4459,7 +4515,7 @@
         <v>166</v>
       </c>
       <c r="AL36" s="8" t="s">
-        <v>74</v>
+        <v>359</v>
       </c>
     </row>
     <row r="37" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -4893,7 +4949,7 @@
         <v>233</v>
       </c>
       <c r="D41" s="8"/>
-      <c r="E41" s="8" t="s">
+      <c r="E41" s="18" t="s">
         <v>234</v>
       </c>
       <c r="F41" s="8" t="s">
@@ -4987,7 +5043,7 @@
         <v>166</v>
       </c>
       <c r="AL41" s="8" t="s">
-        <v>74</v>
+        <v>359</v>
       </c>
     </row>
     <row r="42" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -5098,7 +5154,7 @@
       <c r="C43" s="8" t="s">
         <v>301</v>
       </c>
-      <c r="E43" s="8" t="s">
+      <c r="E43" s="18" t="s">
         <v>302</v>
       </c>
       <c r="F43" s="8" t="s">
@@ -5185,7 +5241,7 @@
         <v>166</v>
       </c>
       <c r="AL43" s="8" t="s">
-        <v>74</v>
+        <v>359</v>
       </c>
     </row>
     <row r="44" spans="1:38" s="8" customFormat="1" x14ac:dyDescent="0.25">
@@ -5206,23 +5262,35 @@
       </c>
       <c r="M44" s="14"/>
       <c r="N44" s="14"/>
+      <c r="O44" s="8" t="s">
+        <v>142</v>
+      </c>
       <c r="P44" s="14"/>
       <c r="Q44" s="15"/>
       <c r="S44" s="15"/>
+      <c r="AL44" s="8" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="45" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A45" s="8" t="s">
         <v>280</v>
       </c>
+      <c r="B45" s="5" t="s">
+        <v>365</v>
+      </c>
       <c r="C45" s="5" t="s">
         <v>348</v>
       </c>
-      <c r="E45" s="5" t="s">
+      <c r="E45" s="8" t="s">
         <v>349</v>
       </c>
       <c r="F45" s="8" t="s">
         <v>157</v>
       </c>
+      <c r="H45" s="5">
+        <v>1921437014</v>
+      </c>
       <c r="I45" s="5">
         <v>1410167293</v>
       </c>
@@ -5244,20 +5312,184 @@
       <c r="Q45" s="7">
         <v>5112217939</v>
       </c>
+      <c r="R45" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="S45" s="7">
+        <v>1731570644612</v>
+      </c>
+      <c r="T45" s="8" t="s">
+        <v>171</v>
+      </c>
+      <c r="U45" s="8" t="s">
+        <v>216</v>
+      </c>
       <c r="V45" s="5" t="s">
         <v>351</v>
       </c>
+      <c r="W45" s="5" t="s">
+        <v>361</v>
+      </c>
+      <c r="X45" s="5">
+        <v>1946653418</v>
+      </c>
+      <c r="Y45" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="Z45" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="AA45" s="5" t="s">
+        <v>362</v>
+      </c>
+      <c r="AB45" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="AC45" s="5" t="s">
+        <v>363</v>
+      </c>
+      <c r="AD45" s="5" t="s">
+        <v>363</v>
+      </c>
+      <c r="AE45" s="5" t="s">
+        <v>361</v>
+      </c>
+      <c r="AF45" s="5" t="s">
+        <v>364</v>
+      </c>
+      <c r="AG45" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AH45" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AI45" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AJ45" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AK45" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AL45" s="8" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="46" spans="1:38" x14ac:dyDescent="0.25">
+      <c r="A46" s="8" t="s">
+        <v>280</v>
+      </c>
+      <c r="B46" s="5" t="s">
+        <v>367</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>366</v>
+      </c>
+      <c r="E46" s="8" t="s">
+        <v>360</v>
+      </c>
+      <c r="F46" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="H46" s="5">
+        <v>1605632547</v>
+      </c>
+      <c r="I46" s="5">
+        <v>1410449332</v>
+      </c>
+      <c r="J46" s="5" t="s">
+        <v>368</v>
+      </c>
+      <c r="K46" s="8">
+        <v>10000</v>
+      </c>
+      <c r="M46" s="6">
+        <v>46174</v>
+      </c>
+      <c r="O46" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="P46" s="6">
+        <v>38475</v>
+      </c>
+      <c r="Q46" s="7">
+        <v>9587105819</v>
+      </c>
+      <c r="V46" s="5" t="s">
+        <v>369</v>
+      </c>
+      <c r="W46" s="5" t="s">
+        <v>370</v>
+      </c>
+      <c r="X46" s="5">
+        <v>1913711156</v>
+      </c>
+      <c r="Y46" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="Z46" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="AA46" s="5" t="s">
+        <v>371</v>
+      </c>
+      <c r="AB46" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="AC46" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="AD46" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="AE46" s="5" t="s">
+        <v>370</v>
+      </c>
+      <c r="AF46" s="5" t="s">
+        <v>373</v>
+      </c>
+      <c r="AG46" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AH46" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AI46" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AJ46" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AK46" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AL46" s="8" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="47" spans="1:38" x14ac:dyDescent="0.25">
+      <c r="E47" s="8"/>
+    </row>
+    <row r="48" spans="1:38" x14ac:dyDescent="0.25">
+      <c r="E48" s="8"/>
+    </row>
+    <row r="49" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E49" s="8"/>
+    </row>
+    <row r="50" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E50" s="8"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
+  <conditionalFormatting sqref="C1:C1048576">
+    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="J1:J1048576">
-    <cfRule type="duplicateValues" dxfId="2" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q1:Q1048576">
-    <cfRule type="duplicateValues" dxfId="1" priority="3"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="3"/>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
feat: add CreateEventModal and DeleteConfirmModal components for event management
- Implemented CreateEventModal for creating and editing events with form validation and data fetching.
- Added DeleteConfirmModal for confirming event deletions with loading state.
- Integrated modals into ZoomInPage with state management for showing/hiding modals and handling submissions.
- Updated translations for new modal functionalities and search fields.
- Enhanced API error handling to provide more informative error messages.
</commit_message>
<xml_diff>
--- a/backend/data/emplyoees.xlsx
+++ b/backend/data/emplyoees.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\emil\projects\Orange-Flow-Next-Js\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D828ED5-2DF0-44DB-B4BB-491A0EF9ACAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4C004EB-3C03-43AB-970C-16AFD7561D60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AL$46</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -1287,7 +1286,15 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -5483,13 +5490,13 @@
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:J1048576">
-    <cfRule type="duplicateValues" dxfId="1" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q1:Q1048576">
-    <cfRule type="duplicateValues" dxfId="0" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="3"/>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
feat: add endpoint to link employees to users and implement employee-user linking logic
</commit_message>
<xml_diff>
--- a/backend/data/emplyoees.xlsx
+++ b/backend/data/emplyoees.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\emil\projects\Orange-Flow-Next-Js\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4C004EB-3C03-43AB-970C-16AFD7561D60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91014247-F187-4B65-B4B8-45CFB4CBB7A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AL$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AL$47</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="867" uniqueCount="374">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="885" uniqueCount="378">
   <si>
     <t>DMS_CODE</t>
   </si>
@@ -1161,6 +1161,18 @@
   </si>
   <si>
     <t>Onufa</t>
+  </si>
+  <si>
+    <t>MYMVAI01SUP02</t>
+  </si>
+  <si>
+    <t>ruhulamin</t>
+  </si>
+  <si>
+    <t>MYMVAI01SUP04</t>
+  </si>
+  <si>
+    <t>Ruhul Amin</t>
   </si>
 </sst>
 </file>
@@ -1286,15 +1298,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="3">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1629,7 +1633,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AL50"/>
+  <dimension ref="A1:AL51"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.5703125" style="5" bestFit="1" customWidth="1"/>
@@ -5258,6 +5262,9 @@
       <c r="B44" s="16" t="s">
         <v>347</v>
       </c>
+      <c r="C44" s="8" t="s">
+        <v>374</v>
+      </c>
       <c r="E44" s="8" t="s">
         <v>346</v>
       </c>
@@ -5267,103 +5274,78 @@
       <c r="H44" s="8">
         <v>1911229913</v>
       </c>
-      <c r="M44" s="14"/>
+      <c r="I44" s="8">
+        <v>1923909896</v>
+      </c>
+      <c r="M44" s="14">
+        <v>43709</v>
+      </c>
       <c r="N44" s="14"/>
       <c r="O44" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="P44" s="14"/>
-      <c r="Q44" s="15"/>
+      <c r="P44" s="14">
+        <v>29571</v>
+      </c>
+      <c r="Q44" s="15">
+        <v>4201594605</v>
+      </c>
       <c r="S44" s="15"/>
+      <c r="AG44" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AH44" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AI44" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AJ44" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AK44" s="8" t="s">
+        <v>166</v>
+      </c>
       <c r="AL44" s="8" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="45" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A45" s="8" t="s">
-        <v>280</v>
-      </c>
-      <c r="B45" s="5" t="s">
-        <v>365</v>
-      </c>
-      <c r="C45" s="5" t="s">
-        <v>348</v>
+    <row r="45" spans="1:38" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="9" t="s">
+        <v>278</v>
+      </c>
+      <c r="B45" s="16" t="s">
+        <v>375</v>
+      </c>
+      <c r="C45" s="8" t="s">
+        <v>376</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>349</v>
+        <v>377</v>
       </c>
       <c r="F45" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="H45" s="5">
-        <v>1921437014</v>
-      </c>
-      <c r="I45" s="5">
-        <v>1410167293</v>
-      </c>
-      <c r="J45" s="5" t="s">
-        <v>350</v>
-      </c>
-      <c r="K45" s="8">
-        <v>10000</v>
-      </c>
-      <c r="M45" s="6">
-        <v>46174</v>
-      </c>
+        <v>284</v>
+      </c>
+      <c r="H45" s="8">
+        <v>1911266077</v>
+      </c>
+      <c r="I45" s="8">
+        <v>1911266077</v>
+      </c>
+      <c r="M45" s="14">
+        <v>44378</v>
+      </c>
+      <c r="N45" s="14"/>
       <c r="O45" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="P45" s="6">
-        <v>35929</v>
-      </c>
-      <c r="Q45" s="7">
-        <v>5112217939</v>
-      </c>
-      <c r="R45" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="S45" s="7">
-        <v>1731570644612</v>
-      </c>
-      <c r="T45" s="8" t="s">
-        <v>171</v>
-      </c>
-      <c r="U45" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="V45" s="5" t="s">
-        <v>351</v>
-      </c>
-      <c r="W45" s="5" t="s">
-        <v>361</v>
-      </c>
-      <c r="X45" s="5">
-        <v>1946653418</v>
-      </c>
-      <c r="Y45" s="5" t="s">
-        <v>238</v>
-      </c>
-      <c r="Z45" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="AA45" s="5" t="s">
-        <v>362</v>
-      </c>
-      <c r="AB45" s="8" t="s">
-        <v>148</v>
-      </c>
-      <c r="AC45" s="5" t="s">
-        <v>363</v>
-      </c>
-      <c r="AD45" s="5" t="s">
-        <v>363</v>
-      </c>
-      <c r="AE45" s="5" t="s">
-        <v>361</v>
-      </c>
-      <c r="AF45" s="5" t="s">
-        <v>364</v>
-      </c>
+      <c r="P45" s="14">
+        <v>35495</v>
+      </c>
+      <c r="Q45" s="15">
+        <v>1.9974815471E+16</v>
+      </c>
+      <c r="S45" s="15"/>
       <c r="AG45" s="8" t="s">
         <v>166</v>
       </c>
@@ -5388,25 +5370,25 @@
         <v>280</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>366</v>
+        <v>348</v>
       </c>
       <c r="E46" s="8" t="s">
-        <v>360</v>
+        <v>349</v>
       </c>
       <c r="F46" s="8" t="s">
         <v>157</v>
       </c>
       <c r="H46" s="5">
-        <v>1605632547</v>
+        <v>1921437014</v>
       </c>
       <c r="I46" s="5">
-        <v>1410449332</v>
+        <v>1410167293</v>
       </c>
       <c r="J46" s="5" t="s">
-        <v>368</v>
+        <v>350</v>
       </c>
       <c r="K46" s="8">
         <v>10000</v>
@@ -5418,19 +5400,31 @@
         <v>142</v>
       </c>
       <c r="P46" s="6">
-        <v>38475</v>
+        <v>35929</v>
       </c>
       <c r="Q46" s="7">
-        <v>9587105819</v>
+        <v>5112217939</v>
+      </c>
+      <c r="R46" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="S46" s="7">
+        <v>1731570644612</v>
+      </c>
+      <c r="T46" s="8" t="s">
+        <v>171</v>
+      </c>
+      <c r="U46" s="8" t="s">
+        <v>216</v>
       </c>
       <c r="V46" s="5" t="s">
-        <v>369</v>
+        <v>351</v>
       </c>
       <c r="W46" s="5" t="s">
-        <v>370</v>
+        <v>361</v>
       </c>
       <c r="X46" s="5">
-        <v>1913711156</v>
+        <v>1946653418</v>
       </c>
       <c r="Y46" s="5" t="s">
         <v>238</v>
@@ -5439,22 +5433,22 @@
         <v>146</v>
       </c>
       <c r="AA46" s="5" t="s">
-        <v>371</v>
+        <v>362</v>
       </c>
       <c r="AB46" s="8" t="s">
-        <v>162</v>
+        <v>148</v>
       </c>
       <c r="AC46" s="5" t="s">
-        <v>372</v>
+        <v>363</v>
       </c>
       <c r="AD46" s="5" t="s">
-        <v>372</v>
+        <v>363</v>
       </c>
       <c r="AE46" s="5" t="s">
-        <v>370</v>
+        <v>361</v>
       </c>
       <c r="AF46" s="5" t="s">
-        <v>373</v>
+        <v>364</v>
       </c>
       <c r="AG46" s="8" t="s">
         <v>166</v>
@@ -5476,7 +5470,96 @@
       </c>
     </row>
     <row r="47" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="E47" s="8"/>
+      <c r="A47" s="8" t="s">
+        <v>280</v>
+      </c>
+      <c r="B47" s="5" t="s">
+        <v>367</v>
+      </c>
+      <c r="C47" s="5" t="s">
+        <v>366</v>
+      </c>
+      <c r="E47" s="8" t="s">
+        <v>360</v>
+      </c>
+      <c r="F47" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="H47" s="5">
+        <v>1605632547</v>
+      </c>
+      <c r="I47" s="5">
+        <v>1410449332</v>
+      </c>
+      <c r="J47" s="5" t="s">
+        <v>368</v>
+      </c>
+      <c r="K47" s="8">
+        <v>10000</v>
+      </c>
+      <c r="M47" s="6">
+        <v>46174</v>
+      </c>
+      <c r="O47" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="P47" s="6">
+        <v>38475</v>
+      </c>
+      <c r="Q47" s="7">
+        <v>9587105819</v>
+      </c>
+      <c r="V47" s="5" t="s">
+        <v>369</v>
+      </c>
+      <c r="W47" s="5" t="s">
+        <v>370</v>
+      </c>
+      <c r="X47" s="5">
+        <v>1913711156</v>
+      </c>
+      <c r="Y47" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="Z47" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="AA47" s="5" t="s">
+        <v>371</v>
+      </c>
+      <c r="AB47" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="AC47" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="AD47" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="AE47" s="5" t="s">
+        <v>370</v>
+      </c>
+      <c r="AF47" s="5" t="s">
+        <v>373</v>
+      </c>
+      <c r="AG47" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AH47" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AI47" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AJ47" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AK47" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AL47" s="8" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="48" spans="1:38" x14ac:dyDescent="0.25">
       <c r="E48" s="8"/>
@@ -5487,16 +5570,19 @@
     <row r="50" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E50" s="8"/>
     </row>
+    <row r="51" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E51" s="8"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:J1048576">
-    <cfRule type="duplicateValues" dxfId="2" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q1:Q1048576">
-    <cfRule type="duplicateValues" dxfId="1" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="3"/>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
feat: implement live report export functionality with ExcelJS and enhance report layout
</commit_message>
<xml_diff>
--- a/backend/data/emplyoees.xlsx
+++ b/backend/data/emplyoees.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\emil\projects\Orange-Flow-Next-Js\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91014247-F187-4B65-B4B8-45CFB4CBB7A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3F8C858-AD95-458F-8C59-C167FD5E17E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="885" uniqueCount="378">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="905" uniqueCount="385">
   <si>
     <t>DMS_CODE</t>
   </si>
@@ -1173,6 +1173,27 @@
   </si>
   <si>
     <t>Ruhul Amin</t>
+  </si>
+  <si>
+    <t>Jasim Uddin Suman</t>
+  </si>
+  <si>
+    <t>Bhairab Bazar</t>
+  </si>
+  <si>
+    <t>Suraiya</t>
+  </si>
+  <si>
+    <t>O-</t>
+  </si>
+  <si>
+    <t>Bhairabpur Dokkhin Para, Bhairab, Kishoreganj.</t>
+  </si>
+  <si>
+    <t>Rofiqul Islam</t>
+  </si>
+  <si>
+    <t>Firoza Akter</t>
   </si>
 </sst>
 </file>
@@ -1238,7 +1259,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1293,6 +1314,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3294,7 +3318,7 @@
       <c r="D22" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="E22" s="9" t="s">
+      <c r="E22" s="19" t="s">
         <v>118</v>
       </c>
       <c r="F22" s="9" t="s">
@@ -3312,7 +3336,9 @@
       <c r="M22" s="10">
         <v>45870</v>
       </c>
-      <c r="N22" s="10"/>
+      <c r="N22" s="10">
+        <v>46203</v>
+      </c>
       <c r="O22" s="9" t="s">
         <v>142</v>
       </c>
@@ -5562,7 +5588,84 @@
       </c>
     </row>
     <row r="48" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="E48" s="8"/>
+      <c r="A48" s="9" t="s">
+        <v>278</v>
+      </c>
+      <c r="E48" s="8" t="s">
+        <v>378</v>
+      </c>
+      <c r="F48" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="H48" s="5">
+        <v>1966727374</v>
+      </c>
+      <c r="I48" s="9">
+        <v>1935597976</v>
+      </c>
+      <c r="M48" s="6">
+        <v>46204</v>
+      </c>
+      <c r="O48" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="P48" s="6">
+        <v>28705</v>
+      </c>
+      <c r="Q48" s="7">
+        <v>2400568289</v>
+      </c>
+      <c r="V48" s="5" t="s">
+        <v>379</v>
+      </c>
+      <c r="W48" s="5" t="s">
+        <v>380</v>
+      </c>
+      <c r="X48" s="5">
+        <v>1937936060</v>
+      </c>
+      <c r="Y48" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="Z48" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="AA48" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="AB48" s="5" t="s">
+        <v>381</v>
+      </c>
+      <c r="AC48" s="5" t="s">
+        <v>382</v>
+      </c>
+      <c r="AD48" s="5" t="s">
+        <v>382</v>
+      </c>
+      <c r="AE48" s="5" t="s">
+        <v>383</v>
+      </c>
+      <c r="AF48" s="5" t="s">
+        <v>384</v>
+      </c>
+      <c r="AG48" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AH48" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AI48" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AJ48" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AK48" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AL48" s="8" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="49" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E49" s="8"/>

</xml_diff>

<commit_message>
feat: refactor exportLiveReport function to streamline data handling and improve layout
</commit_message>
<xml_diff>
--- a/backend/data/emplyoees.xlsx
+++ b/backend/data/emplyoees.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\emil\projects\Orange-Flow-Next-Js\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3F8C858-AD95-458F-8C59-C167FD5E17E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{777A2B3F-0D66-44B2-B43B-620F16C8B914}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="905" uniqueCount="385">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="928" uniqueCount="396">
   <si>
     <t>DMS_CODE</t>
   </si>
@@ -1194,6 +1194,39 @@
   </si>
   <si>
     <t>Firoza Akter</t>
+  </si>
+  <si>
+    <t>MER-RYZBRB0132</t>
+  </si>
+  <si>
+    <t>Kutub Uddin Ripu</t>
+  </si>
+  <si>
+    <t>R648521</t>
+  </si>
+  <si>
+    <t>R344412</t>
+  </si>
+  <si>
+    <t>Itna</t>
+  </si>
+  <si>
+    <t>Tamim Ahmed</t>
+  </si>
+  <si>
+    <t>Cousin</t>
+  </si>
+  <si>
+    <t>Itna High School</t>
+  </si>
+  <si>
+    <t>Laim Pasha, Itna, Kishoreganj.</t>
+  </si>
+  <si>
+    <t>Romjan Ali</t>
+  </si>
+  <si>
+    <t>Rohima Khatun</t>
   </si>
 </sst>
 </file>
@@ -5603,6 +5636,9 @@
       <c r="I48" s="9">
         <v>1935597976</v>
       </c>
+      <c r="J48" s="5" t="s">
+        <v>388</v>
+      </c>
       <c r="M48" s="6">
         <v>46204</v>
       </c>
@@ -5667,13 +5703,96 @@
         <v>74</v>
       </c>
     </row>
-    <row r="49" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E49" s="8"/>
+    <row r="49" spans="1:38" x14ac:dyDescent="0.25">
+      <c r="A49" s="8" t="s">
+        <v>280</v>
+      </c>
+      <c r="C49" s="5" t="s">
+        <v>385</v>
+      </c>
+      <c r="E49" s="8" t="s">
+        <v>386</v>
+      </c>
+      <c r="F49" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="H49" s="5">
+        <v>1410490086</v>
+      </c>
+      <c r="I49" s="5">
+        <v>1410490086</v>
+      </c>
+      <c r="J49" s="5" t="s">
+        <v>387</v>
+      </c>
+      <c r="M49" s="6">
+        <v>46204</v>
+      </c>
+      <c r="O49" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="P49" s="6">
+        <v>32854</v>
+      </c>
+      <c r="Q49" s="7">
+        <v>4813386925537</v>
+      </c>
+      <c r="V49" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="W49" s="5" t="s">
+        <v>390</v>
+      </c>
+      <c r="X49" s="5">
+        <v>1796245290</v>
+      </c>
+      <c r="Y49" s="5" t="s">
+        <v>391</v>
+      </c>
+      <c r="Z49" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="AA49" s="5" t="s">
+        <v>392</v>
+      </c>
+      <c r="AB49" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="AC49" s="5" t="s">
+        <v>393</v>
+      </c>
+      <c r="AD49" s="5" t="s">
+        <v>393</v>
+      </c>
+      <c r="AE49" s="5" t="s">
+        <v>394</v>
+      </c>
+      <c r="AF49" s="5" t="s">
+        <v>395</v>
+      </c>
+      <c r="AG49" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AH49" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AI49" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AJ49" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AK49" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AL49" s="8" t="s">
+        <v>74</v>
+      </c>
     </row>
-    <row r="50" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:38" x14ac:dyDescent="0.25">
       <c r="E50" s="8"/>
     </row>
-    <row r="51" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:38" x14ac:dyDescent="0.25">
       <c r="E51" s="8"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: enhance RSO targets retrieval with pagination and filtering options, update UI components for better user experience
</commit_message>
<xml_diff>
--- a/backend/data/emplyoees.xlsx
+++ b/backend/data/emplyoees.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\emil\projects\Orange-Flow-Next-Js\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{777A2B3F-0D66-44B2-B43B-620F16C8B914}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D3D77F0-161B-4922-86C1-4E6D33D870C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AL$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AL$49</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="928" uniqueCount="396">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="929" uniqueCount="397">
   <si>
     <t>DMS_CODE</t>
   </si>
@@ -1227,6 +1227,9 @@
   </si>
   <si>
     <t>Rohima Khatun</t>
+  </si>
+  <si>
+    <t>MER-MYMVAI0125</t>
   </si>
 </sst>
 </file>
@@ -5624,6 +5627,9 @@
       <c r="A48" s="9" t="s">
         <v>278</v>
       </c>
+      <c r="C48" s="5" t="s">
+        <v>396</v>
+      </c>
       <c r="E48" s="8" t="s">
         <v>378</v>
       </c>

</xml_diff>

<commit_message>
feat: add optional SR number to Employee model and update related components
</commit_message>
<xml_diff>
--- a/backend/data/emplyoees.xlsx
+++ b/backend/data/emplyoees.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\emil\projects\Orange-Flow-Next-Js\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D3D77F0-161B-4922-86C1-4E6D33D870C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81868FA2-C0E0-4C32-9D0D-42A67BCCF058}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AL$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AM$49</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="929" uniqueCount="397">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="955" uniqueCount="423">
   <si>
     <t>DMS_CODE</t>
   </si>
@@ -1230,6 +1230,84 @@
   </si>
   <si>
     <t>MER-MYMVAI0125</t>
+  </si>
+  <si>
+    <t>SR_NO</t>
+  </si>
+  <si>
+    <t>SR-26</t>
+  </si>
+  <si>
+    <t>SR-04</t>
+  </si>
+  <si>
+    <t>SR-05</t>
+  </si>
+  <si>
+    <t>SR-24</t>
+  </si>
+  <si>
+    <t>SR-10</t>
+  </si>
+  <si>
+    <t>SR-11</t>
+  </si>
+  <si>
+    <t>SR-12</t>
+  </si>
+  <si>
+    <t>SR-23</t>
+  </si>
+  <si>
+    <t>SR-25</t>
+  </si>
+  <si>
+    <t>SR-20</t>
+  </si>
+  <si>
+    <t>SR-21</t>
+  </si>
+  <si>
+    <t>SR-01</t>
+  </si>
+  <si>
+    <t>SR-02</t>
+  </si>
+  <si>
+    <t>SR-03</t>
+  </si>
+  <si>
+    <t>SR-06</t>
+  </si>
+  <si>
+    <t>SR-08</t>
+  </si>
+  <si>
+    <t>SR-07</t>
+  </si>
+  <si>
+    <t>SR-14</t>
+  </si>
+  <si>
+    <t>SR-15</t>
+  </si>
+  <si>
+    <t>SR-16</t>
+  </si>
+  <si>
+    <t>SR-17</t>
+  </si>
+  <si>
+    <t>SR-18</t>
+  </si>
+  <si>
+    <t>SR-19</t>
+  </si>
+  <si>
+    <t>SR-09</t>
+  </si>
+  <si>
+    <t>SR-13</t>
   </si>
 </sst>
 </file>
@@ -1693,7 +1771,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AL51"/>
+  <dimension ref="A1:AM51"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.5703125" style="5" bestFit="1" customWidth="1"/>
@@ -1702,41 +1780,42 @@
     <col min="4" max="4" width="13.28515625" style="5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="25.140625" style="5" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.42578125" style="5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.28515625" style="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15" style="5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="24.42578125" style="5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.7109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.85546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.28515625" style="6" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.5703125" style="6" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.42578125" style="5" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10" style="6" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="18.28515625" style="7" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.7109375" style="7" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="15.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="18.7109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="15.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="37.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="39.7109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="13.85546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="16.85546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="38.28515625" style="5" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="14.85546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="29" max="30" width="53.42578125" style="5" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="16.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="18.7109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="27.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="28.7109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="12.7109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="8" style="5" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="16.85546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="8" style="5" bestFit="1" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="5"/>
+    <col min="7" max="7" width="10.42578125" style="5" customWidth="1"/>
+    <col min="8" max="8" width="14.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15" style="5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="24.42578125" style="5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7.7109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.28515625" style="6" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.5703125" style="6" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.42578125" style="5" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10" style="6" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.28515625" style="7" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="12.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="16.7109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="15.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="18.7109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="15.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="37.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="39.7109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="13.85546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="16.85546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="38.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="14.85546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="30" max="31" width="53.42578125" style="5" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="16.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="18.7109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="27.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="28.7109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="12.7109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="8" style="5" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="16.85546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="8" style="5" bestFit="1" customWidth="1"/>
+    <col min="40" max="16384" width="9.140625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>277</v>
       </c>
@@ -1756,103 +1835,106 @@
         <v>2</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>397</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="O1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="R1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="T1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="AF1" s="1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="AG1" s="1" t="s">
+      <c r="AH1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="AH1" s="1" t="s">
+      <c r="AI1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="AI1" s="1" t="s">
+      <c r="AJ1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="AJ1" s="1" t="s">
+      <c r="AK1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="AK1" s="1" t="s">
+      <c r="AL1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="AL1" s="1" t="s">
+      <c r="AM1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:39" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>278</v>
       </c>
@@ -1871,46 +1953,46 @@
       <c r="F2" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="G2" s="9">
+      <c r="G2" s="9" t="s">
+        <v>405</v>
+      </c>
+      <c r="H2" s="9">
         <v>1409944001</v>
       </c>
-      <c r="H2" s="9">
+      <c r="I2" s="9">
         <v>1831949395</v>
       </c>
-      <c r="I2" s="9">
+      <c r="J2" s="9">
         <v>1935593311</v>
       </c>
-      <c r="J2" s="9" t="s">
+      <c r="K2" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="K2" s="9">
+      <c r="L2" s="9">
         <v>8000</v>
       </c>
-      <c r="L2" s="9" t="s">
+      <c r="M2" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="M2" s="10">
+      <c r="N2" s="10">
         <v>45505</v>
       </c>
-      <c r="N2" s="10"/>
-      <c r="O2" s="9" t="s">
+      <c r="O2" s="10"/>
+      <c r="P2" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="P2" s="10">
+      <c r="Q2" s="10">
         <v>37174</v>
       </c>
-      <c r="Q2" s="9" t="s">
+      <c r="R2" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="R2" s="9" t="s">
+      <c r="S2" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="S2" s="11">
+      <c r="T2" s="11">
         <v>1731580054121</v>
       </c>
-      <c r="AG2" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH2" s="8" t="s">
         <v>166</v>
       </c>
@@ -1923,11 +2005,14 @@
       <c r="AK2" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="AL2" s="9" t="s">
+      <c r="AL2" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM2" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="3" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:39" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>278</v>
       </c>
@@ -1946,46 +2031,46 @@
       <c r="F3" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="G3" s="9">
+      <c r="G3" s="9" t="s">
+        <v>406</v>
+      </c>
+      <c r="H3" s="9">
         <v>1908441954</v>
       </c>
-      <c r="H3" s="9">
+      <c r="I3" s="9">
         <v>1911916176</v>
       </c>
-      <c r="I3" s="9">
+      <c r="J3" s="9">
         <v>1935591829</v>
       </c>
-      <c r="J3" s="9" t="s">
+      <c r="K3" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="K3" s="9">
+      <c r="L3" s="9">
         <v>9260</v>
       </c>
-      <c r="L3" s="9" t="s">
+      <c r="M3" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="M3" s="10">
+      <c r="N3" s="10">
         <v>43132</v>
       </c>
-      <c r="N3" s="10"/>
-      <c r="O3" s="9" t="s">
+      <c r="O3" s="10"/>
+      <c r="P3" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="P3" s="10">
+      <c r="Q3" s="10">
         <v>34856</v>
       </c>
-      <c r="Q3" s="9" t="s">
+      <c r="R3" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="R3" s="9" t="s">
+      <c r="S3" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="S3" s="11">
+      <c r="T3" s="11">
         <v>1731030011186</v>
       </c>
-      <c r="AG3" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH3" s="8" t="s">
         <v>166</v>
       </c>
@@ -1998,11 +2083,14 @@
       <c r="AK3" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="AL3" s="9" t="s">
+      <c r="AL3" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM3" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="4" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:39" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>278</v>
       </c>
@@ -2021,43 +2109,43 @@
       <c r="F4" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="G4" s="9">
+      <c r="G4" s="9" t="s">
+        <v>407</v>
+      </c>
+      <c r="H4" s="9">
         <v>1908441955</v>
       </c>
-      <c r="I4" s="9">
+      <c r="J4" s="9">
         <v>1935591837</v>
       </c>
-      <c r="J4" s="9" t="s">
+      <c r="K4" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="K4" s="9">
+      <c r="L4" s="9">
         <v>9662</v>
       </c>
-      <c r="L4" s="9" t="s">
+      <c r="M4" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="M4" s="10">
+      <c r="N4" s="10">
         <v>43160</v>
       </c>
-      <c r="N4" s="10"/>
-      <c r="O4" s="9" t="s">
+      <c r="O4" s="10"/>
+      <c r="P4" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="P4" s="10">
+      <c r="Q4" s="10">
         <v>29571</v>
       </c>
-      <c r="Q4" s="9" t="s">
+      <c r="R4" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="R4" s="9" t="s">
+      <c r="S4" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="S4" s="11">
+      <c r="T4" s="11">
         <v>1731510158618</v>
       </c>
-      <c r="AG4" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH4" s="8" t="s">
         <v>166</v>
       </c>
@@ -2070,11 +2158,14 @@
       <c r="AK4" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="AL4" s="9" t="s">
+      <c r="AL4" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM4" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="5" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:39" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
         <v>278</v>
       </c>
@@ -2090,44 +2181,44 @@
       <c r="F5" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="G5" s="9">
+      <c r="G5" s="9" t="s">
+        <v>408</v>
+      </c>
+      <c r="H5" s="9">
         <v>1915270101</v>
       </c>
-      <c r="H5" s="9">
+      <c r="I5" s="9">
         <v>1401607080</v>
       </c>
-      <c r="I5" s="9">
+      <c r="J5" s="9">
         <v>1935591856</v>
       </c>
-      <c r="J5" s="9" t="s">
+      <c r="K5" s="9" t="s">
         <v>355</v>
       </c>
-      <c r="K5" s="9">
+      <c r="L5" s="9">
         <v>9500</v>
       </c>
-      <c r="L5" s="9" t="s">
+      <c r="M5" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="M5" s="10">
+      <c r="N5" s="10">
         <v>46174</v>
       </c>
-      <c r="N5" s="10"/>
-      <c r="O5" s="9" t="s">
+      <c r="O5" s="10"/>
+      <c r="P5" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="P5" s="10">
+      <c r="Q5" s="10">
         <v>32538</v>
       </c>
-      <c r="Q5" s="9">
+      <c r="R5" s="9">
         <v>6850022234</v>
       </c>
-      <c r="R5" s="9" t="s">
+      <c r="S5" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="S5" s="11"/>
-      <c r="AG5" s="8" t="s">
-        <v>166</v>
-      </c>
+      <c r="T5" s="11"/>
       <c r="AH5" s="8" t="s">
         <v>166</v>
       </c>
@@ -2140,11 +2231,14 @@
       <c r="AK5" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="AL5" s="9" t="s">
+      <c r="AL5" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM5" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="6" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:39" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>278</v>
       </c>
@@ -2163,43 +2257,43 @@
       <c r="F6" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="G6" s="9">
+      <c r="G6" s="9" t="s">
+        <v>409</v>
+      </c>
+      <c r="H6" s="9">
         <v>1915270102</v>
       </c>
-      <c r="I6" s="9">
+      <c r="J6" s="9">
         <v>1935592000</v>
       </c>
-      <c r="J6" s="9" t="s">
+      <c r="K6" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="K6" s="9">
+      <c r="L6" s="9">
         <v>8500</v>
       </c>
-      <c r="L6" s="9" t="s">
+      <c r="M6" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="M6" s="10">
+      <c r="N6" s="10">
         <v>45840</v>
       </c>
-      <c r="N6" s="10"/>
-      <c r="O6" s="9" t="s">
+      <c r="O6" s="10"/>
+      <c r="P6" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="P6" s="10">
+      <c r="Q6" s="10">
         <v>38178</v>
       </c>
-      <c r="Q6" s="9" t="s">
+      <c r="R6" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="R6" s="9" t="s">
+      <c r="S6" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="S6" s="11">
+      <c r="T6" s="11">
         <v>1731580357541</v>
       </c>
-      <c r="AG6" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH6" s="8" t="s">
         <v>166</v>
       </c>
@@ -2212,11 +2306,14 @@
       <c r="AK6" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="AL6" s="9" t="s">
+      <c r="AL6" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM6" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:39" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
         <v>278</v>
       </c>
@@ -2232,46 +2329,46 @@
       <c r="F7" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="G7" s="9">
+      <c r="G7" s="9" t="s">
+        <v>410</v>
+      </c>
+      <c r="H7" s="9">
         <v>1409944003</v>
       </c>
-      <c r="H7" s="9">
+      <c r="I7" s="9">
         <v>1813862410</v>
       </c>
-      <c r="I7" s="9">
+      <c r="J7" s="9">
         <v>1935593312</v>
       </c>
-      <c r="J7" s="9" t="s">
+      <c r="K7" s="9" t="s">
         <v>353</v>
       </c>
-      <c r="K7" s="9">
+      <c r="L7" s="9">
         <v>8500</v>
       </c>
-      <c r="L7" s="9" t="s">
+      <c r="M7" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="M7" s="10">
+      <c r="N7" s="10">
         <v>46174</v>
       </c>
-      <c r="N7" s="10"/>
-      <c r="O7" s="9" t="s">
+      <c r="O7" s="10"/>
+      <c r="P7" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="P7" s="10">
+      <c r="Q7" s="10">
         <v>38716</v>
       </c>
-      <c r="Q7" s="9" t="s">
+      <c r="R7" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="R7" s="9" t="s">
+      <c r="S7" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="S7" s="11">
+      <c r="T7" s="11">
         <v>2311030477929</v>
       </c>
-      <c r="AG7" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH7" s="8" t="s">
         <v>166</v>
       </c>
@@ -2284,11 +2381,14 @@
       <c r="AK7" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="AL7" s="9" t="s">
+      <c r="AL7" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM7" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="8" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:39" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>278</v>
       </c>
@@ -2307,84 +2407,84 @@
       <c r="F8" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="G8" s="9">
+      <c r="G8" s="9" t="s">
+        <v>411</v>
+      </c>
+      <c r="H8" s="9">
         <v>1915270103</v>
       </c>
-      <c r="H8" s="9">
+      <c r="I8" s="9">
         <v>1764864677</v>
       </c>
-      <c r="I8" s="9">
+      <c r="J8" s="9">
         <v>1935591914</v>
       </c>
-      <c r="J8" s="9" t="s">
+      <c r="K8" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="K8" s="9">
+      <c r="L8" s="9">
         <v>9500</v>
       </c>
-      <c r="L8" s="9" t="s">
+      <c r="M8" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="M8" s="10">
+      <c r="N8" s="10">
         <v>46143</v>
       </c>
-      <c r="N8" s="10"/>
-      <c r="O8" s="9" t="s">
+      <c r="O8" s="10"/>
+      <c r="P8" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="P8" s="10">
+      <c r="Q8" s="10">
         <v>38512</v>
       </c>
-      <c r="Q8" s="8">
+      <c r="R8" s="8">
         <v>7824872522</v>
       </c>
-      <c r="R8" s="12" t="s">
+      <c r="S8" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="S8" s="13">
+      <c r="T8" s="13">
         <v>2311030553506</v>
       </c>
-      <c r="V8" s="9" t="s">
+      <c r="W8" s="9" t="s">
         <v>143</v>
       </c>
-      <c r="W8" s="9" t="s">
+      <c r="X8" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="X8" s="9">
+      <c r="Y8" s="9">
         <v>1742609199</v>
       </c>
-      <c r="Y8" s="9" t="s">
+      <c r="Z8" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="Z8" s="9" t="s">
+      <c r="AA8" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="AA8" s="9" t="s">
+      <c r="AB8" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="AB8" s="9" t="s">
+      <c r="AC8" s="9" t="s">
         <v>148</v>
-      </c>
-      <c r="AC8" s="9" t="s">
-        <v>149</v>
       </c>
       <c r="AD8" s="9" t="s">
         <v>149</v>
       </c>
       <c r="AE8" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="AF8" s="9" t="s">
         <v>150</v>
       </c>
-      <c r="AF8" s="9" t="s">
+      <c r="AG8" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="AG8" s="9" t="s">
+      <c r="AH8" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="AH8" s="9">
+      <c r="AI8" s="9">
         <v>9000</v>
-      </c>
-      <c r="AI8" s="9" t="s">
-        <v>153</v>
       </c>
       <c r="AJ8" s="9" t="s">
         <v>153</v>
@@ -2393,10 +2493,13 @@
         <v>153</v>
       </c>
       <c r="AL8" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="AM8" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="9" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:39" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>278</v>
       </c>
@@ -2415,43 +2518,43 @@
       <c r="F9" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="G9" s="9">
+      <c r="G9" s="9" t="s">
+        <v>412</v>
+      </c>
+      <c r="H9" s="9">
         <v>1915270106</v>
       </c>
-      <c r="I9" s="9">
+      <c r="J9" s="9">
         <v>1935591815</v>
       </c>
-      <c r="J9" s="9" t="s">
+      <c r="K9" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="K9" s="9">
+      <c r="L9" s="9">
         <v>8500</v>
       </c>
-      <c r="L9" s="9" t="s">
+      <c r="M9" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="M9" s="10">
+      <c r="N9" s="10">
         <v>45909</v>
       </c>
-      <c r="N9" s="10"/>
-      <c r="O9" s="9" t="s">
+      <c r="O9" s="10"/>
+      <c r="P9" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="P9" s="10">
+      <c r="Q9" s="10">
         <v>37448</v>
       </c>
-      <c r="Q9" s="9" t="s">
+      <c r="R9" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="R9" s="9" t="s">
+      <c r="S9" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="S9" s="11">
+      <c r="T9" s="11">
         <v>2311030377356</v>
       </c>
-      <c r="AG9" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH9" s="8" t="s">
         <v>166</v>
       </c>
@@ -2464,11 +2567,14 @@
       <c r="AK9" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="AL9" s="9" t="s">
+      <c r="AL9" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM9" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="10" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:39" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
         <v>278</v>
       </c>
@@ -2487,46 +2593,46 @@
       <c r="F10" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="G10" s="9">
+      <c r="G10" s="9" t="s">
+        <v>413</v>
+      </c>
+      <c r="H10" s="9">
         <v>1915300196</v>
       </c>
-      <c r="H10" s="9">
+      <c r="I10" s="9">
         <v>1917509966</v>
       </c>
-      <c r="I10" s="9">
+      <c r="J10" s="9">
         <v>1935591797</v>
       </c>
-      <c r="J10" s="9" t="s">
+      <c r="K10" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="K10" s="9">
+      <c r="L10" s="9">
         <v>8500</v>
       </c>
-      <c r="L10" s="9" t="s">
+      <c r="M10" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="M10" s="10">
+      <c r="N10" s="10">
         <v>45873</v>
       </c>
-      <c r="N10" s="10"/>
-      <c r="O10" s="9" t="s">
+      <c r="O10" s="10"/>
+      <c r="P10" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="P10" s="10">
+      <c r="Q10" s="10">
         <v>36526</v>
       </c>
-      <c r="Q10" s="9" t="s">
+      <c r="R10" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="R10" s="9" t="s">
+      <c r="S10" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="S10" s="11">
+      <c r="T10" s="11">
         <v>2311580115485</v>
       </c>
-      <c r="AG10" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH10" s="8" t="s">
         <v>166</v>
       </c>
@@ -2539,11 +2645,14 @@
       <c r="AK10" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="AL10" s="9" t="s">
+      <c r="AL10" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM10" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="11" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:39" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>278</v>
       </c>
@@ -2562,43 +2671,43 @@
       <c r="F11" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="G11" s="9">
+      <c r="G11" s="9" t="s">
+        <v>414</v>
+      </c>
+      <c r="H11" s="9">
         <v>1937600512</v>
       </c>
-      <c r="I11" s="9">
+      <c r="J11" s="9">
         <v>1935591796</v>
       </c>
-      <c r="J11" s="9" t="s">
+      <c r="K11" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="K11" s="9">
+      <c r="L11" s="9">
         <v>8500</v>
       </c>
-      <c r="L11" s="9" t="s">
+      <c r="M11" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="M11" s="10">
+      <c r="N11" s="10">
         <v>45976</v>
       </c>
-      <c r="N11" s="10"/>
-      <c r="O11" s="9" t="s">
+      <c r="O11" s="10"/>
+      <c r="P11" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="P11" s="10">
+      <c r="Q11" s="10">
         <v>38644</v>
       </c>
-      <c r="Q11" s="9" t="s">
+      <c r="R11" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="R11" s="9" t="s">
+      <c r="S11" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="S11" s="11">
+      <c r="T11" s="11">
         <v>1731580447892</v>
       </c>
-      <c r="AG11" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH11" s="8" t="s">
         <v>166</v>
       </c>
@@ -2611,11 +2720,14 @@
       <c r="AK11" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="AL11" s="9" t="s">
+      <c r="AL11" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM11" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="12" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:39" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
         <v>278</v>
       </c>
@@ -2634,46 +2746,46 @@
       <c r="F12" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="G12" s="9">
+      <c r="G12" s="9" t="s">
+        <v>415</v>
+      </c>
+      <c r="H12" s="9">
         <v>1984217911</v>
       </c>
-      <c r="H12" s="9">
+      <c r="I12" s="9">
         <v>1775222954</v>
       </c>
-      <c r="I12" s="9">
+      <c r="J12" s="9">
         <v>1935591918</v>
       </c>
-      <c r="J12" s="9" t="s">
+      <c r="K12" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="K12" s="9">
+      <c r="L12" s="9">
         <v>8500</v>
       </c>
-      <c r="L12" s="9" t="s">
+      <c r="M12" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="M12" s="10">
+      <c r="N12" s="10">
         <v>45909</v>
       </c>
-      <c r="N12" s="10"/>
-      <c r="O12" s="9" t="s">
+      <c r="O12" s="10"/>
+      <c r="P12" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="P12" s="10">
+      <c r="Q12" s="10">
         <v>35458</v>
       </c>
-      <c r="Q12" s="9" t="s">
+      <c r="R12" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="R12" s="9" t="s">
+      <c r="S12" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="S12" s="11">
+      <c r="T12" s="11">
         <v>2311030047576</v>
       </c>
-      <c r="AG12" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH12" s="8" t="s">
         <v>166</v>
       </c>
@@ -2686,11 +2798,14 @@
       <c r="AK12" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="AL12" s="9" t="s">
+      <c r="AL12" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM12" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="13" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:39" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>278</v>
       </c>
@@ -2709,43 +2824,43 @@
       <c r="F13" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="G13" s="9">
+      <c r="G13" s="9" t="s">
+        <v>416</v>
+      </c>
+      <c r="H13" s="9">
         <v>1984217912</v>
       </c>
-      <c r="I13" s="9">
+      <c r="J13" s="9">
         <v>1935591999</v>
       </c>
-      <c r="J13" s="9" t="s">
+      <c r="K13" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="K13" s="9">
+      <c r="L13" s="9">
         <v>8500</v>
       </c>
-      <c r="L13" s="9" t="s">
+      <c r="M13" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="M13" s="10">
+      <c r="N13" s="10">
         <v>45965</v>
       </c>
-      <c r="N13" s="10"/>
-      <c r="O13" s="9" t="s">
+      <c r="O13" s="10"/>
+      <c r="P13" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="P13" s="10">
+      <c r="Q13" s="10">
         <v>38845</v>
       </c>
-      <c r="Q13" s="9" t="s">
+      <c r="R13" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="R13" s="9" t="s">
+      <c r="S13" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="S13" s="11">
+      <c r="T13" s="11">
         <v>2311030422596</v>
       </c>
-      <c r="AG13" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH13" s="8" t="s">
         <v>166</v>
       </c>
@@ -2758,11 +2873,14 @@
       <c r="AK13" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="AL13" s="9" t="s">
+      <c r="AL13" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM13" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="14" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:39" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
         <v>278</v>
       </c>
@@ -2781,46 +2899,46 @@
       <c r="F14" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="G14" s="9">
+      <c r="G14" s="9" t="s">
+        <v>417</v>
+      </c>
+      <c r="H14" s="9">
         <v>1984220363</v>
       </c>
-      <c r="H14" s="9">
+      <c r="I14" s="9">
         <v>1620502971</v>
       </c>
-      <c r="I14" s="9">
+      <c r="J14" s="9">
         <v>1935591917</v>
       </c>
-      <c r="J14" s="9" t="s">
+      <c r="K14" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="K14" s="9">
+      <c r="L14" s="9">
         <v>8500</v>
       </c>
-      <c r="L14" s="9" t="s">
+      <c r="M14" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="M14" s="10">
+      <c r="N14" s="10">
         <v>45748</v>
       </c>
-      <c r="N14" s="10"/>
-      <c r="O14" s="9" t="s">
+      <c r="O14" s="10"/>
+      <c r="P14" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="P14" s="10">
+      <c r="Q14" s="10">
         <v>33898</v>
       </c>
-      <c r="Q14" s="9" t="s">
+      <c r="R14" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="R14" s="9" t="s">
+      <c r="S14" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="S14" s="11">
+      <c r="T14" s="11">
         <v>1731580062730</v>
       </c>
-      <c r="AG14" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH14" s="8" t="s">
         <v>166</v>
       </c>
@@ -2833,11 +2951,14 @@
       <c r="AK14" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="AL14" s="9" t="s">
+      <c r="AL14" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM14" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="15" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:39" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>278</v>
       </c>
@@ -2856,46 +2977,46 @@
       <c r="F15" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="G15" s="9">
+      <c r="G15" s="9" t="s">
+        <v>418</v>
+      </c>
+      <c r="H15" s="9">
         <v>1984220364</v>
       </c>
-      <c r="H15" s="9">
+      <c r="I15" s="9">
         <v>1997616187</v>
       </c>
-      <c r="I15" s="9">
+      <c r="J15" s="9">
         <v>1935591855</v>
       </c>
-      <c r="J15" s="9" t="s">
+      <c r="K15" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="K15" s="9">
+      <c r="L15" s="9">
         <v>8500</v>
       </c>
-      <c r="L15" s="9" t="s">
+      <c r="M15" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="M15" s="10">
+      <c r="N15" s="10">
         <v>45999</v>
       </c>
-      <c r="N15" s="10"/>
-      <c r="O15" s="9" t="s">
+      <c r="O15" s="10"/>
+      <c r="P15" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="P15" s="10">
+      <c r="Q15" s="10">
         <v>37991</v>
       </c>
-      <c r="Q15" s="9" t="s">
+      <c r="R15" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="R15" s="9" t="s">
+      <c r="S15" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="S15" s="11">
+      <c r="T15" s="11">
         <v>1737348886514</v>
       </c>
-      <c r="AG15" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH15" s="8" t="s">
         <v>166</v>
       </c>
@@ -2908,11 +3029,14 @@
       <c r="AK15" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="AL15" s="9" t="s">
+      <c r="AL15" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM15" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="16" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:39" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
         <v>278</v>
       </c>
@@ -2931,46 +3055,46 @@
       <c r="F16" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="G16" s="9">
+      <c r="G16" s="9" t="s">
+        <v>419</v>
+      </c>
+      <c r="H16" s="9">
         <v>1984220365</v>
       </c>
-      <c r="H16" s="9">
+      <c r="I16" s="9">
         <v>1970772132</v>
       </c>
-      <c r="I16" s="9">
+      <c r="J16" s="9">
         <v>1935591913</v>
       </c>
-      <c r="J16" s="9" t="s">
+      <c r="K16" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="K16" s="9">
+      <c r="L16" s="9">
         <v>8404</v>
       </c>
-      <c r="L16" s="9" t="s">
+      <c r="M16" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="M16" s="10">
+      <c r="N16" s="10">
         <v>43709</v>
       </c>
-      <c r="N16" s="10"/>
-      <c r="O16" s="9" t="s">
+      <c r="O16" s="10"/>
+      <c r="P16" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="P16" s="10">
+      <c r="Q16" s="10">
         <v>36114</v>
       </c>
-      <c r="Q16" s="9" t="s">
+      <c r="R16" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="R16" s="9" t="s">
+      <c r="S16" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="S16" s="11">
+      <c r="T16" s="11">
         <v>1731030011132</v>
       </c>
-      <c r="AG16" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH16" s="8" t="s">
         <v>166</v>
       </c>
@@ -2983,11 +3107,14 @@
       <c r="AK16" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="AL16" s="9" t="s">
+      <c r="AL16" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM16" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="17" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:39" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>278</v>
       </c>
@@ -3006,46 +3133,46 @@
       <c r="F17" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="G17" s="9">
+      <c r="G17" s="9" t="s">
+        <v>420</v>
+      </c>
+      <c r="H17" s="9">
         <v>1984220366</v>
       </c>
-      <c r="H17" s="9">
+      <c r="I17" s="9">
         <v>1915343494</v>
       </c>
-      <c r="I17" s="9">
+      <c r="J17" s="9">
         <v>1935592054</v>
       </c>
-      <c r="J17" s="9" t="s">
+      <c r="K17" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="K17" s="9">
+      <c r="L17" s="9">
         <v>8580</v>
       </c>
-      <c r="L17" s="9" t="s">
+      <c r="M17" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="M17" s="10">
+      <c r="N17" s="10">
         <v>44470</v>
       </c>
-      <c r="N17" s="10"/>
-      <c r="O17" s="9" t="s">
+      <c r="O17" s="10"/>
+      <c r="P17" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="P17" s="10">
+      <c r="Q17" s="10">
         <v>36318</v>
       </c>
-      <c r="Q17" s="9" t="s">
+      <c r="R17" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="R17" s="9" t="s">
+      <c r="S17" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="S17" s="11">
+      <c r="T17" s="11">
         <v>1731510173296</v>
       </c>
-      <c r="AG17" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH17" s="8" t="s">
         <v>166</v>
       </c>
@@ -3058,11 +3185,14 @@
       <c r="AK17" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="AL17" s="9" t="s">
+      <c r="AL17" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM17" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="18" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:39" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
         <v>278</v>
       </c>
@@ -3081,43 +3211,43 @@
       <c r="F18" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="G18" s="9">
+      <c r="G18" s="9" t="s">
+        <v>421</v>
+      </c>
+      <c r="H18" s="9">
         <v>1986646474</v>
       </c>
-      <c r="I18" s="9">
+      <c r="J18" s="9">
         <v>1935592053</v>
       </c>
-      <c r="J18" s="9" t="s">
+      <c r="K18" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="K18" s="9">
+      <c r="L18" s="9">
         <v>9350</v>
       </c>
-      <c r="L18" s="9" t="s">
+      <c r="M18" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="M18" s="10">
+      <c r="N18" s="10">
         <v>45444</v>
       </c>
-      <c r="N18" s="10"/>
-      <c r="O18" s="9" t="s">
+      <c r="O18" s="10"/>
+      <c r="P18" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="P18" s="10">
+      <c r="Q18" s="10">
         <v>32174</v>
       </c>
-      <c r="Q18" s="9" t="s">
+      <c r="R18" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="R18" s="9" t="s">
+      <c r="S18" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="S18" s="11">
+      <c r="T18" s="11">
         <v>7017332507958</v>
       </c>
-      <c r="AG18" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH18" s="8" t="s">
         <v>166</v>
       </c>
@@ -3130,11 +3260,14 @@
       <c r="AK18" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="AL18" s="9" t="s">
+      <c r="AL18" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM18" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="19" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:39" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>278</v>
       </c>
@@ -3153,46 +3286,46 @@
       <c r="F19" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="G19" s="9">
+      <c r="G19" s="9" t="s">
+        <v>422</v>
+      </c>
+      <c r="H19" s="9">
         <v>1986686880</v>
       </c>
-      <c r="H19" s="9">
+      <c r="I19" s="9">
         <v>1924303333</v>
       </c>
-      <c r="I19" s="9">
+      <c r="J19" s="9">
         <v>1935591915</v>
       </c>
-      <c r="J19" s="9" t="s">
+      <c r="K19" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="K19" s="9">
+      <c r="L19" s="9">
         <v>8500</v>
       </c>
-      <c r="L19" s="9" t="s">
+      <c r="M19" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="M19" s="10">
+      <c r="N19" s="10">
         <v>46023</v>
       </c>
-      <c r="N19" s="10"/>
-      <c r="O19" s="9" t="s">
+      <c r="O19" s="10"/>
+      <c r="P19" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="P19" s="10">
+      <c r="Q19" s="10">
         <v>36557</v>
       </c>
-      <c r="Q19" s="9" t="s">
+      <c r="R19" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="R19" s="9" t="s">
+      <c r="S19" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="S19" s="11">
+      <c r="T19" s="11">
         <v>1731030011127</v>
       </c>
-      <c r="AG19" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH19" s="8" t="s">
         <v>166</v>
       </c>
@@ -3205,11 +3338,14 @@
       <c r="AK19" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="AL19" s="9" t="s">
+      <c r="AL19" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM19" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="20" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:39" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
         <v>278</v>
       </c>
@@ -3228,37 +3364,34 @@
       <c r="F20" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="H20" s="9">
+      <c r="I20" s="9">
         <v>1912317878</v>
       </c>
-      <c r="I20" s="9">
+      <c r="J20" s="9">
         <v>1958041930</v>
       </c>
-      <c r="J20" s="9" t="s">
+      <c r="K20" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="M20" s="10">
+      <c r="N20" s="10">
         <v>42370</v>
       </c>
-      <c r="N20" s="10"/>
-      <c r="O20" s="9" t="s">
+      <c r="O20" s="10"/>
+      <c r="P20" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="P20" s="10">
+      <c r="Q20" s="10">
         <v>33675</v>
       </c>
-      <c r="Q20" s="9" t="s">
+      <c r="R20" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="R20" s="9" t="s">
+      <c r="S20" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="S20" s="11">
+      <c r="T20" s="11">
         <v>1731510105407</v>
       </c>
-      <c r="AG20" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH20" s="8" t="s">
         <v>166</v>
       </c>
@@ -3271,11 +3404,14 @@
       <c r="AK20" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="AL20" s="9" t="s">
+      <c r="AL20" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM20" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="21" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:39" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
         <v>278</v>
       </c>
@@ -3294,37 +3430,34 @@
       <c r="F21" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="H21" s="9">
+      <c r="I21" s="9">
         <v>1911626293</v>
       </c>
-      <c r="I21" s="9">
+      <c r="J21" s="9">
         <v>1958041928</v>
       </c>
-      <c r="J21" s="9" t="s">
+      <c r="K21" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="M21" s="10">
+      <c r="N21" s="10">
         <v>41122</v>
       </c>
-      <c r="N21" s="10"/>
-      <c r="O21" s="9" t="s">
+      <c r="O21" s="10"/>
+      <c r="P21" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="P21" s="10">
+      <c r="Q21" s="10">
         <v>30806</v>
       </c>
-      <c r="Q21" s="9" t="s">
+      <c r="R21" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="R21" s="9" t="s">
+      <c r="S21" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="S21" s="11">
+      <c r="T21" s="11">
         <v>1471030170630</v>
       </c>
-      <c r="AG21" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH21" s="8" t="s">
         <v>166</v>
       </c>
@@ -3337,11 +3470,14 @@
       <c r="AK21" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="AL21" s="9" t="s">
+      <c r="AL21" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM21" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="22" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:39" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
         <v>278</v>
       </c>
@@ -3360,39 +3496,36 @@
       <c r="F22" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="H22" s="9">
+      <c r="I22" s="9">
         <v>1711228193</v>
       </c>
-      <c r="I22" s="9">
+      <c r="J22" s="9">
         <v>1935597976</v>
       </c>
-      <c r="J22" s="9" t="s">
+      <c r="K22" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="M22" s="10">
+      <c r="N22" s="10">
         <v>45870</v>
       </c>
-      <c r="N22" s="10">
+      <c r="O22" s="10">
         <v>46203</v>
       </c>
-      <c r="O22" s="9" t="s">
+      <c r="P22" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="P22" s="10">
+      <c r="Q22" s="10">
         <v>30806</v>
       </c>
-      <c r="Q22" s="9">
+      <c r="R22" s="9">
         <v>2860896055</v>
       </c>
-      <c r="R22" s="9" t="s">
+      <c r="S22" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="S22" s="11">
+      <c r="T22" s="11">
         <v>1731030011382</v>
       </c>
-      <c r="AG22" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH22" s="8" t="s">
         <v>166</v>
       </c>
@@ -3405,11 +3538,14 @@
       <c r="AK22" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="AL22" s="9" t="s">
+      <c r="AL22" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM22" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="23" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:39" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
         <v>278</v>
       </c>
@@ -3428,37 +3564,34 @@
       <c r="F23" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="H23" s="9">
+      <c r="I23" s="9">
         <v>1913453027</v>
       </c>
-      <c r="I23" s="9">
+      <c r="J23" s="9">
         <v>1935597774</v>
       </c>
-      <c r="J23" s="9" t="s">
+      <c r="K23" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="M23" s="10">
+      <c r="N23" s="10">
         <v>46054</v>
       </c>
-      <c r="N23" s="10"/>
-      <c r="O23" s="9" t="s">
+      <c r="O23" s="10"/>
+      <c r="P23" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="P23" s="10">
+      <c r="Q23" s="10">
         <v>37337</v>
       </c>
-      <c r="Q23" s="9" t="s">
+      <c r="R23" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="R23" s="9" t="s">
+      <c r="S23" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="S23" s="11">
+      <c r="T23" s="11">
         <v>1731050036178</v>
       </c>
-      <c r="AG23" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH23" s="8" t="s">
         <v>166</v>
       </c>
@@ -3471,11 +3604,14 @@
       <c r="AK23" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="AL23" s="9" t="s">
+      <c r="AL23" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM23" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="24" spans="1:38" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:39" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
         <v>279</v>
       </c>
@@ -3492,26 +3628,28 @@
       <c r="F24" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="G24" s="9">
+      <c r="G24" s="9" t="s">
+        <v>398</v>
+      </c>
+      <c r="H24" s="9">
         <v>1409944002</v>
       </c>
-      <c r="H24" s="9"/>
-      <c r="I24" s="9">
+      <c r="I24" s="9"/>
+      <c r="J24" s="9">
         <v>1935593313</v>
       </c>
-      <c r="J24" s="9" t="s">
+      <c r="K24" s="9" t="s">
         <v>358</v>
       </c>
-      <c r="K24" s="9"/>
       <c r="L24" s="9"/>
-      <c r="M24" s="17"/>
-      <c r="N24" s="10"/>
-      <c r="O24" s="9"/>
-      <c r="P24" s="17"/>
-      <c r="Q24" s="9"/>
+      <c r="M24" s="9"/>
+      <c r="N24" s="17"/>
+      <c r="O24" s="10"/>
+      <c r="P24" s="9"/>
+      <c r="Q24" s="17"/>
       <c r="R24" s="9"/>
-      <c r="S24" s="11"/>
-      <c r="T24" s="9"/>
+      <c r="S24" s="9"/>
+      <c r="T24" s="11"/>
       <c r="U24" s="9"/>
       <c r="V24" s="9"/>
       <c r="W24" s="9"/>
@@ -3524,9 +3662,7 @@
       <c r="AD24" s="9"/>
       <c r="AE24" s="9"/>
       <c r="AF24" s="9"/>
-      <c r="AG24" s="8" t="s">
-        <v>166</v>
-      </c>
+      <c r="AG24" s="9"/>
       <c r="AH24" s="8" t="s">
         <v>166</v>
       </c>
@@ -3539,11 +3675,14 @@
       <c r="AK24" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="AL24" s="9" t="s">
+      <c r="AL24" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM24" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="25" spans="1:38" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:39" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
         <v>279</v>
       </c>
@@ -3562,42 +3701,44 @@
       <c r="F25" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="G25" s="9">
+      <c r="G25" s="9" t="s">
+        <v>399</v>
+      </c>
+      <c r="H25" s="9">
         <v>1915270104</v>
       </c>
-      <c r="H25" s="9"/>
-      <c r="I25" s="9">
+      <c r="I25" s="9"/>
+      <c r="J25" s="9">
         <v>1935591816</v>
       </c>
-      <c r="J25" s="9" t="s">
+      <c r="K25" s="9" t="s">
         <v>246</v>
       </c>
-      <c r="K25" s="9">
+      <c r="L25" s="9">
         <v>7000</v>
       </c>
-      <c r="L25" s="9" t="s">
+      <c r="M25" s="9" t="s">
         <v>242</v>
       </c>
-      <c r="M25" s="17">
+      <c r="N25" s="17">
         <v>45474</v>
       </c>
-      <c r="N25" s="10"/>
-      <c r="O25" s="9" t="s">
+      <c r="O25" s="10"/>
+      <c r="P25" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="P25" s="17">
+      <c r="Q25" s="17">
         <v>38443</v>
       </c>
-      <c r="Q25" s="9" t="s">
+      <c r="R25" s="9" t="s">
         <v>247</v>
       </c>
-      <c r="R25" s="9" t="s">
+      <c r="S25" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="S25" s="11">
+      <c r="T25" s="11">
         <v>2311580121330</v>
       </c>
-      <c r="T25" s="9"/>
       <c r="U25" s="9"/>
       <c r="V25" s="9"/>
       <c r="W25" s="9"/>
@@ -3610,9 +3751,7 @@
       <c r="AD25" s="9"/>
       <c r="AE25" s="9"/>
       <c r="AF25" s="9"/>
-      <c r="AG25" s="8" t="s">
-        <v>166</v>
-      </c>
+      <c r="AG25" s="9"/>
       <c r="AH25" s="8" t="s">
         <v>166</v>
       </c>
@@ -3625,11 +3764,14 @@
       <c r="AK25" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="AL25" s="9" t="s">
+      <c r="AL25" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM25" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="26" spans="1:38" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:39" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
         <v>279</v>
       </c>
@@ -3648,42 +3790,44 @@
       <c r="F26" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="G26" s="9">
+      <c r="G26" s="9" t="s">
+        <v>400</v>
+      </c>
+      <c r="H26" s="9">
         <v>1915270105</v>
       </c>
-      <c r="H26" s="9"/>
-      <c r="I26" s="9">
+      <c r="I26" s="9"/>
+      <c r="J26" s="9">
         <v>1935591916</v>
       </c>
-      <c r="J26" s="9" t="s">
+      <c r="K26" s="9" t="s">
         <v>251</v>
       </c>
-      <c r="K26" s="9">
+      <c r="L26" s="9">
         <v>9500</v>
       </c>
-      <c r="L26" s="9" t="s">
+      <c r="M26" s="9" t="s">
         <v>242</v>
       </c>
-      <c r="M26" s="17">
+      <c r="N26" s="17">
         <v>45909</v>
       </c>
-      <c r="N26" s="10"/>
-      <c r="O26" s="9" t="s">
+      <c r="O26" s="10"/>
+      <c r="P26" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="P26" s="17">
+      <c r="Q26" s="17">
         <v>38952</v>
       </c>
-      <c r="Q26" s="9" t="s">
+      <c r="R26" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="R26" s="9" t="s">
+      <c r="S26" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="S26" s="11">
+      <c r="T26" s="11">
         <v>2311580453888</v>
       </c>
-      <c r="T26" s="9"/>
       <c r="U26" s="9"/>
       <c r="V26" s="9"/>
       <c r="W26" s="9"/>
@@ -3696,9 +3840,7 @@
       <c r="AD26" s="9"/>
       <c r="AE26" s="9"/>
       <c r="AF26" s="9"/>
-      <c r="AG26" s="8" t="s">
-        <v>166</v>
-      </c>
+      <c r="AG26" s="9"/>
       <c r="AH26" s="8" t="s">
         <v>166</v>
       </c>
@@ -3711,11 +3853,14 @@
       <c r="AK26" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="AL26" s="9" t="s">
+      <c r="AL26" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM26" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="27" spans="1:38" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:39" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="9" t="s">
         <v>279</v>
       </c>
@@ -3734,42 +3879,44 @@
       <c r="F27" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="G27" s="9">
+      <c r="G27" s="9" t="s">
+        <v>401</v>
+      </c>
+      <c r="H27" s="9">
         <v>1967042950</v>
       </c>
-      <c r="H27" s="9"/>
-      <c r="I27" s="9">
+      <c r="I27" s="9"/>
+      <c r="J27" s="9">
         <v>1935592484</v>
       </c>
-      <c r="J27" s="9" t="s">
+      <c r="K27" s="9" t="s">
         <v>256</v>
       </c>
-      <c r="K27" s="9">
+      <c r="L27" s="9">
         <v>9500</v>
       </c>
-      <c r="L27" s="9" t="s">
+      <c r="M27" s="9" t="s">
         <v>242</v>
       </c>
-      <c r="M27" s="17">
+      <c r="N27" s="17">
         <v>45909</v>
       </c>
-      <c r="N27" s="10"/>
-      <c r="O27" s="9" t="s">
+      <c r="O27" s="10"/>
+      <c r="P27" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="P27" s="17">
+      <c r="Q27" s="17">
         <v>38688</v>
       </c>
-      <c r="Q27" s="9" t="s">
+      <c r="R27" s="9" t="s">
         <v>257</v>
       </c>
-      <c r="R27" s="9" t="s">
+      <c r="S27" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="S27" s="11">
+      <c r="T27" s="11">
         <v>2311030382527</v>
       </c>
-      <c r="T27" s="9"/>
       <c r="U27" s="9"/>
       <c r="V27" s="9"/>
       <c r="W27" s="9"/>
@@ -3782,9 +3929,7 @@
       <c r="AD27" s="9"/>
       <c r="AE27" s="9"/>
       <c r="AF27" s="9"/>
-      <c r="AG27" s="8" t="s">
-        <v>166</v>
-      </c>
+      <c r="AG27" s="9"/>
       <c r="AH27" s="8" t="s">
         <v>166</v>
       </c>
@@ -3797,11 +3942,14 @@
       <c r="AK27" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="AL27" s="9" t="s">
+      <c r="AL27" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM27" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="28" spans="1:38" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:39" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="9" t="s">
         <v>279</v>
       </c>
@@ -3820,42 +3968,44 @@
       <c r="F28" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="G28" s="9">
+      <c r="G28" s="9" t="s">
+        <v>402</v>
+      </c>
+      <c r="H28" s="9">
         <v>1986686877</v>
       </c>
-      <c r="H28" s="9"/>
-      <c r="I28" s="9">
+      <c r="I28" s="9"/>
+      <c r="J28" s="9">
         <v>1935591836</v>
       </c>
-      <c r="J28" s="9" t="s">
+      <c r="K28" s="9" t="s">
         <v>261</v>
       </c>
-      <c r="K28" s="9">
+      <c r="L28" s="9">
         <v>7000</v>
       </c>
-      <c r="L28" s="9" t="s">
+      <c r="M28" s="9" t="s">
         <v>242</v>
       </c>
-      <c r="M28" s="17">
+      <c r="N28" s="17">
         <v>45658</v>
       </c>
-      <c r="N28" s="10"/>
-      <c r="O28" s="9" t="s">
+      <c r="O28" s="10"/>
+      <c r="P28" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="P28" s="17">
+      <c r="Q28" s="17">
         <v>37483</v>
       </c>
-      <c r="Q28" s="9" t="s">
+      <c r="R28" s="9" t="s">
         <v>262</v>
       </c>
-      <c r="R28" s="9" t="s">
+      <c r="S28" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="S28" s="11">
+      <c r="T28" s="11">
         <v>2311580181156</v>
       </c>
-      <c r="T28" s="9"/>
       <c r="U28" s="9"/>
       <c r="V28" s="9"/>
       <c r="W28" s="9"/>
@@ -3868,9 +4018,7 @@
       <c r="AD28" s="9"/>
       <c r="AE28" s="9"/>
       <c r="AF28" s="9"/>
-      <c r="AG28" s="8" t="s">
-        <v>166</v>
-      </c>
+      <c r="AG28" s="9"/>
       <c r="AH28" s="8" t="s">
         <v>166</v>
       </c>
@@ -3883,11 +4031,14 @@
       <c r="AK28" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="AL28" s="9" t="s">
+      <c r="AL28" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM28" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="29" spans="1:38" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:39" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="9" t="s">
         <v>279</v>
       </c>
@@ -3906,42 +4057,44 @@
       <c r="F29" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="G29" s="9">
+      <c r="G29" s="9" t="s">
+        <v>403</v>
+      </c>
+      <c r="H29" s="9">
         <v>1986686878</v>
       </c>
-      <c r="H29" s="9"/>
-      <c r="I29" s="9">
+      <c r="I29" s="9"/>
+      <c r="J29" s="9">
         <v>1935591828</v>
       </c>
-      <c r="J29" s="9" t="s">
+      <c r="K29" s="9" t="s">
         <v>265</v>
       </c>
-      <c r="K29" s="9">
+      <c r="L29" s="9">
         <v>10500</v>
       </c>
-      <c r="L29" s="9" t="s">
+      <c r="M29" s="9" t="s">
         <v>242</v>
       </c>
-      <c r="M29" s="17">
+      <c r="N29" s="17">
         <v>46027</v>
       </c>
-      <c r="N29" s="10"/>
-      <c r="O29" s="9" t="s">
+      <c r="O29" s="10"/>
+      <c r="P29" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="P29" s="17">
+      <c r="Q29" s="17">
         <v>35286</v>
       </c>
-      <c r="Q29" s="9" t="s">
+      <c r="R29" s="9" t="s">
         <v>266</v>
       </c>
-      <c r="R29" s="9" t="s">
+      <c r="S29" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="S29" s="11">
+      <c r="T29" s="11">
         <v>1731030011244</v>
       </c>
-      <c r="T29" s="9"/>
       <c r="U29" s="9"/>
       <c r="V29" s="9"/>
       <c r="W29" s="9"/>
@@ -3954,9 +4107,7 @@
       <c r="AD29" s="9"/>
       <c r="AE29" s="9"/>
       <c r="AF29" s="9"/>
-      <c r="AG29" s="8" t="s">
-        <v>166</v>
-      </c>
+      <c r="AG29" s="9"/>
       <c r="AH29" s="8" t="s">
         <v>166</v>
       </c>
@@ -3969,11 +4120,14 @@
       <c r="AK29" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="AL29" s="9" t="s">
+      <c r="AL29" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM29" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="30" spans="1:38" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:39" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="9" t="s">
         <v>279</v>
       </c>
@@ -3990,26 +4144,28 @@
       <c r="F30" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="G30" s="9">
+      <c r="G30" s="9" t="s">
+        <v>404</v>
+      </c>
+      <c r="H30" s="9">
         <v>1986686879</v>
       </c>
-      <c r="H30" s="9"/>
-      <c r="I30" s="9">
+      <c r="I30" s="9"/>
+      <c r="J30" s="9">
         <v>1935592119</v>
       </c>
-      <c r="J30" s="9" t="s">
+      <c r="K30" s="9" t="s">
         <v>267</v>
       </c>
-      <c r="K30" s="9"/>
       <c r="L30" s="9"/>
-      <c r="M30" s="17"/>
-      <c r="N30" s="10"/>
-      <c r="O30" s="9"/>
-      <c r="P30" s="17"/>
-      <c r="Q30" s="9"/>
+      <c r="M30" s="9"/>
+      <c r="N30" s="17"/>
+      <c r="O30" s="10"/>
+      <c r="P30" s="9"/>
+      <c r="Q30" s="17"/>
       <c r="R30" s="9"/>
-      <c r="S30" s="11"/>
-      <c r="T30" s="9"/>
+      <c r="S30" s="9"/>
+      <c r="T30" s="11"/>
       <c r="U30" s="9"/>
       <c r="V30" s="9"/>
       <c r="W30" s="9"/>
@@ -4022,9 +4178,7 @@
       <c r="AD30" s="9"/>
       <c r="AE30" s="9"/>
       <c r="AF30" s="9"/>
-      <c r="AG30" s="8" t="s">
-        <v>166</v>
-      </c>
+      <c r="AG30" s="9"/>
       <c r="AH30" s="8" t="s">
         <v>166</v>
       </c>
@@ -4037,11 +4191,14 @@
       <c r="AK30" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="AL30" s="9" t="s">
+      <c r="AL30" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM30" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="31" spans="1:38" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:39" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="9" t="s">
         <v>279</v>
       </c>
@@ -4061,35 +4218,35 @@
         <v>271</v>
       </c>
       <c r="G31" s="9"/>
-      <c r="H31" s="9">
+      <c r="H31" s="9"/>
+      <c r="I31" s="9">
         <v>1611169592</v>
       </c>
-      <c r="I31" s="9">
+      <c r="J31" s="9">
         <v>1999968844</v>
       </c>
-      <c r="J31" s="9" t="s">
+      <c r="K31" s="9" t="s">
         <v>272</v>
       </c>
-      <c r="K31" s="9"/>
       <c r="L31" s="9"/>
-      <c r="M31" s="9">
+      <c r="M31" s="9"/>
+      <c r="N31" s="9">
         <v>45931</v>
       </c>
-      <c r="N31" s="10"/>
-      <c r="O31" s="9"/>
-      <c r="P31" s="9">
+      <c r="O31" s="10"/>
+      <c r="P31" s="9"/>
+      <c r="Q31" s="9">
         <v>31821</v>
       </c>
-      <c r="Q31" s="9" t="s">
+      <c r="R31" s="9" t="s">
         <v>273</v>
       </c>
-      <c r="R31" s="9" t="s">
+      <c r="S31" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="S31" s="9">
+      <c r="T31" s="9">
         <v>2311580467330</v>
       </c>
-      <c r="T31" s="9"/>
       <c r="U31" s="9"/>
       <c r="V31" s="9"/>
       <c r="W31" s="9"/>
@@ -4102,9 +4259,7 @@
       <c r="AD31" s="9"/>
       <c r="AE31" s="9"/>
       <c r="AF31" s="9"/>
-      <c r="AG31" s="8" t="s">
-        <v>166</v>
-      </c>
+      <c r="AG31" s="9"/>
       <c r="AH31" s="8" t="s">
         <v>166</v>
       </c>
@@ -4117,11 +4272,14 @@
       <c r="AK31" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="AL31" s="9" t="s">
+      <c r="AL31" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM31" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="32" spans="1:38" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:39" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="9" t="s">
         <v>279</v>
       </c>
@@ -4140,17 +4298,17 @@
       </c>
       <c r="G32" s="9"/>
       <c r="H32" s="9"/>
-      <c r="I32" s="9">
+      <c r="I32" s="9"/>
+      <c r="J32" s="9">
         <v>1935600928</v>
       </c>
-      <c r="J32" s="9" t="s">
+      <c r="K32" s="9" t="s">
         <v>276</v>
       </c>
-      <c r="K32" s="9"/>
       <c r="L32" s="9"/>
       <c r="M32" s="9"/>
-      <c r="N32" s="10"/>
-      <c r="O32" s="9"/>
+      <c r="N32" s="9"/>
+      <c r="O32" s="10"/>
       <c r="P32" s="9"/>
       <c r="Q32" s="9"/>
       <c r="R32" s="9"/>
@@ -4168,9 +4326,7 @@
       <c r="AD32" s="9"/>
       <c r="AE32" s="9"/>
       <c r="AF32" s="9"/>
-      <c r="AG32" s="8" t="s">
-        <v>166</v>
-      </c>
+      <c r="AG32" s="9"/>
       <c r="AH32" s="8" t="s">
         <v>166</v>
       </c>
@@ -4183,11 +4339,14 @@
       <c r="AK32" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="AL32" s="9" t="s">
+      <c r="AL32" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM32" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="33" spans="1:38" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:39" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="8" t="s">
         <v>280</v>
       </c>
@@ -4206,67 +4365,64 @@
       <c r="F33" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="H33" s="8">
+      <c r="I33" s="8">
         <v>1786080093</v>
       </c>
-      <c r="I33" s="8">
+      <c r="J33" s="8">
         <v>1410678746</v>
       </c>
-      <c r="J33" s="8" t="s">
+      <c r="K33" s="8" t="s">
         <v>158</v>
       </c>
-      <c r="K33" s="8">
+      <c r="L33" s="8">
         <v>10000</v>
       </c>
-      <c r="M33" s="14">
+      <c r="N33" s="14">
         <v>46082</v>
       </c>
-      <c r="N33" s="14"/>
-      <c r="O33" s="8" t="s">
+      <c r="O33" s="14"/>
+      <c r="P33" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="P33" s="14">
+      <c r="Q33" s="14">
         <v>33834</v>
       </c>
-      <c r="Q33" s="15">
+      <c r="R33" s="15">
         <v>6404733260</v>
       </c>
-      <c r="R33" s="8" t="s">
+      <c r="S33" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="S33" s="15">
+      <c r="T33" s="15">
         <v>1731580493357</v>
       </c>
-      <c r="W33" s="8" t="s">
+      <c r="X33" s="8" t="s">
         <v>160</v>
       </c>
-      <c r="X33" s="8">
+      <c r="Y33" s="8">
         <v>1752787879</v>
       </c>
-      <c r="Y33" s="8" t="s">
+      <c r="Z33" s="8" t="s">
         <v>161</v>
       </c>
-      <c r="Z33" s="8" t="s">
+      <c r="AA33" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="AB33" s="8" t="s">
+      <c r="AC33" s="8" t="s">
         <v>162</v>
-      </c>
-      <c r="AC33" s="8" t="s">
-        <v>165</v>
       </c>
       <c r="AD33" s="8" t="s">
         <v>165</v>
       </c>
       <c r="AE33" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="AF33" s="8" t="s">
         <v>163</v>
       </c>
-      <c r="AF33" s="8" t="s">
+      <c r="AG33" s="8" t="s">
         <v>164</v>
       </c>
-      <c r="AG33" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH33" s="8" t="s">
         <v>166</v>
       </c>
@@ -4280,10 +4436,13 @@
         <v>166</v>
       </c>
       <c r="AL33" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM33" s="8" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="34" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:39" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="8" t="s">
         <v>280</v>
       </c>
@@ -4303,74 +4462,72 @@
         <v>157</v>
       </c>
       <c r="G34" s="8"/>
-      <c r="H34" s="8">
-        <v>1410071973</v>
-      </c>
+      <c r="H34" s="8"/>
       <c r="I34" s="8">
         <v>1410071973</v>
       </c>
-      <c r="J34" s="8" t="s">
+      <c r="J34" s="8">
+        <v>1410071973</v>
+      </c>
+      <c r="K34" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="K34" s="8">
+      <c r="L34" s="8">
         <v>10000</v>
       </c>
-      <c r="L34" s="8"/>
-      <c r="M34" s="14">
+      <c r="M34" s="8"/>
+      <c r="N34" s="14">
         <v>46082</v>
       </c>
-      <c r="N34" s="14"/>
-      <c r="O34" s="8" t="s">
+      <c r="O34" s="14"/>
+      <c r="P34" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="P34" s="14">
+      <c r="Q34" s="14">
         <v>32540</v>
       </c>
-      <c r="Q34" s="15">
+      <c r="R34" s="15">
         <v>1314935507162</v>
       </c>
-      <c r="R34" s="8" t="s">
+      <c r="S34" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="S34" s="15">
+      <c r="T34" s="15">
         <v>1731580492738</v>
       </c>
-      <c r="T34" s="8" t="s">
+      <c r="U34" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="U34" s="8"/>
       <c r="V34" s="8"/>
-      <c r="W34" s="8" t="s">
+      <c r="W34" s="8"/>
+      <c r="X34" s="8" t="s">
         <v>172</v>
       </c>
-      <c r="X34" s="8">
+      <c r="Y34" s="8">
         <v>1864929394</v>
       </c>
-      <c r="Y34" s="8" t="s">
+      <c r="Z34" s="8" t="s">
         <v>161</v>
       </c>
-      <c r="Z34" s="8" t="s">
+      <c r="AA34" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="AA34" s="8"/>
-      <c r="AB34" s="8" t="s">
+      <c r="AB34" s="8"/>
+      <c r="AC34" s="8" t="s">
         <v>173</v>
-      </c>
-      <c r="AC34" s="8" t="s">
-        <v>176</v>
       </c>
       <c r="AD34" s="8" t="s">
         <v>176</v>
       </c>
       <c r="AE34" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="AF34" s="8" t="s">
         <v>174</v>
       </c>
-      <c r="AF34" s="8" t="s">
+      <c r="AG34" s="8" t="s">
         <v>175</v>
       </c>
-      <c r="AG34" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH34" s="8" t="s">
         <v>166</v>
       </c>
@@ -4384,10 +4541,13 @@
         <v>166</v>
       </c>
       <c r="AL34" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM34" s="8" t="s">
         <v>359</v>
       </c>
     </row>
-    <row r="35" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:39" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
         <v>280</v>
       </c>
@@ -4407,72 +4567,70 @@
         <v>157</v>
       </c>
       <c r="G35" s="8"/>
-      <c r="H35" s="8">
-        <v>1410240211</v>
-      </c>
+      <c r="H35" s="8"/>
       <c r="I35" s="8">
         <v>1410240211</v>
       </c>
-      <c r="J35" s="8" t="s">
+      <c r="J35" s="8">
+        <v>1410240211</v>
+      </c>
+      <c r="K35" s="8" t="s">
         <v>180</v>
       </c>
-      <c r="K35" s="8">
+      <c r="L35" s="8">
         <v>10000</v>
       </c>
-      <c r="L35" s="8"/>
-      <c r="M35" s="14">
+      <c r="M35" s="8"/>
+      <c r="N35" s="14">
         <v>45971</v>
       </c>
-      <c r="N35" s="14"/>
-      <c r="O35" s="8" t="s">
+      <c r="O35" s="14"/>
+      <c r="P35" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="P35" s="14">
+      <c r="Q35" s="14">
         <v>1</v>
       </c>
-      <c r="Q35" s="15">
+      <c r="R35" s="15">
         <v>2863545949</v>
       </c>
-      <c r="R35" s="8" t="s">
+      <c r="S35" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="S35" s="15">
+      <c r="T35" s="15">
         <v>1731050292189</v>
       </c>
-      <c r="T35" s="8"/>
       <c r="U35" s="8"/>
       <c r="V35" s="8"/>
-      <c r="W35" s="8" t="s">
+      <c r="W35" s="8"/>
+      <c r="X35" s="8" t="s">
         <v>181</v>
       </c>
-      <c r="X35" s="8">
+      <c r="Y35" s="8">
         <v>1407911493</v>
       </c>
-      <c r="Y35" s="8" t="s">
+      <c r="Z35" s="8" t="s">
         <v>161</v>
       </c>
-      <c r="Z35" s="8" t="s">
+      <c r="AA35" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="AA35" s="8"/>
-      <c r="AB35" s="8" t="s">
+      <c r="AB35" s="8"/>
+      <c r="AC35" s="8" t="s">
         <v>182</v>
-      </c>
-      <c r="AC35" s="8" t="s">
-        <v>185</v>
       </c>
       <c r="AD35" s="8" t="s">
         <v>185</v>
       </c>
       <c r="AE35" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="AF35" s="8" t="s">
         <v>183</v>
       </c>
-      <c r="AF35" s="8" t="s">
+      <c r="AG35" s="8" t="s">
         <v>184</v>
       </c>
-      <c r="AG35" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH35" s="8" t="s">
         <v>166</v>
       </c>
@@ -4486,10 +4644,13 @@
         <v>166</v>
       </c>
       <c r="AL35" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM35" s="8" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="36" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:39" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="8" t="s">
         <v>280</v>
       </c>
@@ -4509,72 +4670,70 @@
         <v>157</v>
       </c>
       <c r="G36" s="8"/>
-      <c r="H36" s="8">
+      <c r="H36" s="8"/>
+      <c r="I36" s="8">
         <v>1917787990</v>
       </c>
-      <c r="I36" s="8">
+      <c r="J36" s="8">
         <v>1410436602</v>
       </c>
-      <c r="J36" s="8" t="s">
+      <c r="K36" s="8" t="s">
         <v>189</v>
       </c>
-      <c r="K36" s="8">
+      <c r="L36" s="8">
         <v>10000</v>
       </c>
-      <c r="L36" s="8"/>
-      <c r="M36" s="14">
+      <c r="M36" s="8"/>
+      <c r="N36" s="14">
         <v>45971</v>
       </c>
-      <c r="N36" s="14"/>
-      <c r="O36" s="8" t="s">
+      <c r="O36" s="14"/>
+      <c r="P36" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="P36" s="14">
+      <c r="Q36" s="14">
         <v>31595</v>
       </c>
-      <c r="Q36" s="15">
+      <c r="R36" s="15">
         <v>4813347971938</v>
       </c>
-      <c r="R36" s="8" t="s">
+      <c r="S36" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="S36" s="15">
+      <c r="T36" s="15">
         <v>2311580489016</v>
       </c>
-      <c r="T36" s="8"/>
       <c r="U36" s="8"/>
       <c r="V36" s="8"/>
-      <c r="W36" s="8" t="s">
+      <c r="W36" s="8"/>
+      <c r="X36" s="8" t="s">
         <v>190</v>
       </c>
-      <c r="X36" s="8">
+      <c r="Y36" s="8">
         <v>1730797404</v>
       </c>
-      <c r="Y36" s="8" t="s">
+      <c r="Z36" s="8" t="s">
         <v>161</v>
       </c>
-      <c r="Z36" s="8" t="s">
+      <c r="AA36" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="AA36" s="8"/>
-      <c r="AB36" s="8" t="s">
+      <c r="AB36" s="8"/>
+      <c r="AC36" s="8" t="s">
         <v>191</v>
-      </c>
-      <c r="AC36" s="8" t="s">
-        <v>194</v>
       </c>
       <c r="AD36" s="8" t="s">
         <v>194</v>
       </c>
       <c r="AE36" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="AF36" s="8" t="s">
         <v>192</v>
       </c>
-      <c r="AF36" s="8" t="s">
+      <c r="AG36" s="8" t="s">
         <v>193</v>
       </c>
-      <c r="AG36" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH36" s="8" t="s">
         <v>166</v>
       </c>
@@ -4588,10 +4747,13 @@
         <v>166</v>
       </c>
       <c r="AL36" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM36" s="8" t="s">
         <v>359</v>
       </c>
     </row>
-    <row r="37" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:39" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="8" t="s">
         <v>280</v>
       </c>
@@ -4611,72 +4773,70 @@
         <v>157</v>
       </c>
       <c r="G37" s="8"/>
-      <c r="H37" s="8">
+      <c r="H37" s="8"/>
+      <c r="I37" s="8">
         <v>1305213723</v>
       </c>
-      <c r="I37" s="8">
+      <c r="J37" s="8">
         <v>1410213723</v>
       </c>
-      <c r="J37" s="8" t="s">
+      <c r="K37" s="8" t="s">
         <v>198</v>
       </c>
-      <c r="K37" s="8">
+      <c r="L37" s="8">
         <v>10000</v>
       </c>
-      <c r="L37" s="8"/>
-      <c r="M37" s="14">
+      <c r="M37" s="8"/>
+      <c r="N37" s="14">
         <v>46054</v>
       </c>
-      <c r="N37" s="14"/>
-      <c r="O37" s="8" t="s">
+      <c r="O37" s="14"/>
+      <c r="P37" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="P37" s="14">
+      <c r="Q37" s="14">
         <v>38161</v>
       </c>
-      <c r="Q37" s="15">
+      <c r="R37" s="15">
         <v>1042040244</v>
       </c>
-      <c r="R37" s="8" t="s">
+      <c r="S37" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="S37" s="15">
+      <c r="T37" s="15">
         <v>2311580512005</v>
       </c>
-      <c r="T37" s="8"/>
       <c r="U37" s="8"/>
       <c r="V37" s="8"/>
-      <c r="W37" s="8" t="s">
+      <c r="W37" s="8"/>
+      <c r="X37" s="8" t="s">
         <v>199</v>
       </c>
-      <c r="X37" s="8">
+      <c r="Y37" s="8">
         <v>1782371767</v>
       </c>
-      <c r="Y37" s="8" t="s">
+      <c r="Z37" s="8" t="s">
         <v>161</v>
       </c>
-      <c r="Z37" s="8" t="s">
+      <c r="AA37" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="AA37" s="8"/>
-      <c r="AB37" s="8" t="s">
+      <c r="AB37" s="8"/>
+      <c r="AC37" s="8" t="s">
         <v>200</v>
-      </c>
-      <c r="AC37" s="8" t="s">
-        <v>203</v>
       </c>
       <c r="AD37" s="8" t="s">
         <v>203</v>
       </c>
       <c r="AE37" s="8" t="s">
+        <v>203</v>
+      </c>
+      <c r="AF37" s="8" t="s">
         <v>201</v>
       </c>
-      <c r="AF37" s="8" t="s">
+      <c r="AG37" s="8" t="s">
         <v>202</v>
       </c>
-      <c r="AG37" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH37" s="8" t="s">
         <v>166</v>
       </c>
@@ -4690,10 +4850,13 @@
         <v>166</v>
       </c>
       <c r="AL37" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM37" s="8" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="38" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:39" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="8" t="s">
         <v>280</v>
       </c>
@@ -4713,72 +4876,70 @@
         <v>157</v>
       </c>
       <c r="G38" s="8"/>
-      <c r="H38" s="8">
+      <c r="H38" s="8"/>
+      <c r="I38" s="8">
         <v>1990757830</v>
       </c>
-      <c r="I38" s="8">
+      <c r="J38" s="8">
         <v>1410173774</v>
       </c>
-      <c r="J38" s="8" t="s">
+      <c r="K38" s="8" t="s">
         <v>207</v>
       </c>
-      <c r="K38" s="8">
+      <c r="L38" s="8">
         <v>10000</v>
       </c>
-      <c r="L38" s="8"/>
-      <c r="M38" s="14">
+      <c r="M38" s="8"/>
+      <c r="N38" s="14">
         <v>46054</v>
       </c>
-      <c r="N38" s="14"/>
-      <c r="O38" s="8" t="s">
+      <c r="O38" s="14"/>
+      <c r="P38" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="P38" s="14">
+      <c r="Q38" s="14">
         <v>33970</v>
       </c>
-      <c r="Q38" s="15">
+      <c r="R38" s="15">
         <v>2824445262</v>
       </c>
-      <c r="R38" s="8" t="s">
+      <c r="S38" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="S38" s="15">
+      <c r="T38" s="15">
         <v>7017344002631</v>
       </c>
-      <c r="T38" s="8"/>
       <c r="U38" s="8"/>
       <c r="V38" s="8"/>
-      <c r="W38" s="8" t="s">
+      <c r="W38" s="8"/>
+      <c r="X38" s="8" t="s">
         <v>208</v>
       </c>
-      <c r="X38" s="8">
+      <c r="Y38" s="8">
         <v>1925717710</v>
       </c>
-      <c r="Y38" s="8" t="s">
+      <c r="Z38" s="8" t="s">
         <v>209</v>
       </c>
-      <c r="Z38" s="8" t="s">
+      <c r="AA38" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="AA38" s="8"/>
-      <c r="AB38" s="8" t="s">
+      <c r="AB38" s="8"/>
+      <c r="AC38" s="8" t="s">
         <v>162</v>
-      </c>
-      <c r="AC38" s="8" t="s">
-        <v>212</v>
       </c>
       <c r="AD38" s="8" t="s">
         <v>212</v>
       </c>
       <c r="AE38" s="8" t="s">
+        <v>212</v>
+      </c>
+      <c r="AF38" s="8" t="s">
         <v>210</v>
       </c>
-      <c r="AF38" s="8" t="s">
+      <c r="AG38" s="8" t="s">
         <v>211</v>
       </c>
-      <c r="AG38" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH38" s="8" t="s">
         <v>166</v>
       </c>
@@ -4792,10 +4953,13 @@
         <v>166</v>
       </c>
       <c r="AL38" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM38" s="8" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="39" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:39" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="8" t="s">
         <v>280</v>
       </c>
@@ -4813,80 +4977,78 @@
         <v>157</v>
       </c>
       <c r="G39" s="8"/>
-      <c r="H39" s="8">
+      <c r="H39" s="8"/>
+      <c r="I39" s="8">
         <v>1763122889</v>
       </c>
-      <c r="I39" s="8">
+      <c r="J39" s="8">
         <v>1410720313</v>
       </c>
-      <c r="J39" s="8" t="s">
+      <c r="K39" s="8" t="s">
         <v>215</v>
       </c>
-      <c r="K39" s="8">
+      <c r="L39" s="8">
         <v>10000</v>
       </c>
-      <c r="L39" s="8"/>
-      <c r="M39" s="14">
+      <c r="M39" s="8"/>
+      <c r="N39" s="14">
         <v>46143</v>
       </c>
-      <c r="N39" s="14"/>
-      <c r="O39" s="8" t="s">
+      <c r="O39" s="14"/>
+      <c r="P39" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="P39" s="14">
+      <c r="Q39" s="14">
         <v>36906</v>
       </c>
-      <c r="Q39" s="15">
+      <c r="R39" s="15">
         <v>8263476999</v>
       </c>
-      <c r="R39" s="8" t="s">
+      <c r="S39" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="S39" s="15">
+      <c r="T39" s="15">
         <v>1731580441218</v>
       </c>
-      <c r="T39" s="8" t="s">
+      <c r="U39" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="U39" s="8" t="s">
+      <c r="V39" s="8" t="s">
         <v>216</v>
       </c>
-      <c r="V39" s="8" t="s">
+      <c r="W39" s="8" t="s">
         <v>217</v>
       </c>
-      <c r="W39" s="8" t="s">
+      <c r="X39" s="8" t="s">
         <v>218</v>
       </c>
-      <c r="X39" s="8">
+      <c r="Y39" s="8">
         <v>1325533299</v>
       </c>
-      <c r="Y39" s="8" t="s">
+      <c r="Z39" s="8" t="s">
         <v>161</v>
       </c>
-      <c r="Z39" s="8" t="s">
+      <c r="AA39" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="AA39" s="8" t="s">
+      <c r="AB39" s="8" t="s">
         <v>219</v>
       </c>
-      <c r="AB39" s="8" t="s">
+      <c r="AC39" s="8" t="s">
         <v>148</v>
-      </c>
-      <c r="AC39" s="8" t="s">
-        <v>222</v>
       </c>
       <c r="AD39" s="8" t="s">
         <v>222</v>
       </c>
       <c r="AE39" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="AF39" s="8" t="s">
         <v>220</v>
       </c>
-      <c r="AF39" s="8" t="s">
+      <c r="AG39" s="8" t="s">
         <v>221</v>
       </c>
-      <c r="AG39" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH39" s="8" t="s">
         <v>166</v>
       </c>
@@ -4900,10 +5062,13 @@
         <v>166</v>
       </c>
       <c r="AL39" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM39" s="8" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="40" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:39" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="8" t="s">
         <v>280</v>
       </c>
@@ -4921,80 +5086,78 @@
         <v>157</v>
       </c>
       <c r="G40" s="8"/>
-      <c r="H40" s="8">
+      <c r="H40" s="8"/>
+      <c r="I40" s="8">
         <v>1984397910</v>
       </c>
-      <c r="I40" s="8">
+      <c r="J40" s="8">
         <v>1410031485</v>
       </c>
-      <c r="J40" s="8" t="s">
+      <c r="K40" s="8" t="s">
         <v>225</v>
       </c>
-      <c r="K40" s="8">
+      <c r="L40" s="8">
         <v>10000</v>
       </c>
-      <c r="L40" s="8"/>
-      <c r="M40" s="14">
+      <c r="M40" s="8"/>
+      <c r="N40" s="14">
         <v>46143</v>
       </c>
-      <c r="N40" s="14"/>
-      <c r="O40" s="8" t="s">
+      <c r="O40" s="14"/>
+      <c r="P40" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="P40" s="14">
+      <c r="Q40" s="14">
         <v>31902</v>
       </c>
-      <c r="Q40" s="15">
+      <c r="R40" s="15">
         <v>5546839951</v>
       </c>
-      <c r="R40" s="8" t="s">
+      <c r="S40" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="S40" s="15">
+      <c r="T40" s="15">
         <v>1731580504974</v>
       </c>
-      <c r="T40" s="8" t="s">
+      <c r="U40" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="U40" s="8" t="s">
+      <c r="V40" s="8" t="s">
         <v>216</v>
       </c>
-      <c r="V40" s="8" t="s">
+      <c r="W40" s="8" t="s">
         <v>226</v>
       </c>
-      <c r="W40" s="8" t="s">
+      <c r="X40" s="8" t="s">
         <v>227</v>
       </c>
-      <c r="X40" s="8">
+      <c r="Y40" s="8">
         <v>1812206330</v>
       </c>
-      <c r="Y40" s="8" t="s">
+      <c r="Z40" s="8" t="s">
         <v>209</v>
       </c>
-      <c r="Z40" s="8" t="s">
+      <c r="AA40" s="8" t="s">
         <v>229</v>
       </c>
-      <c r="AA40" s="8" t="s">
+      <c r="AB40" s="8" t="s">
         <v>228</v>
       </c>
-      <c r="AB40" s="8" t="s">
+      <c r="AC40" s="8" t="s">
         <v>162</v>
-      </c>
-      <c r="AC40" s="8" t="s">
-        <v>232</v>
       </c>
       <c r="AD40" s="8" t="s">
         <v>232</v>
       </c>
       <c r="AE40" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="AF40" s="8" t="s">
         <v>230</v>
       </c>
-      <c r="AF40" s="8" t="s">
+      <c r="AG40" s="8" t="s">
         <v>231</v>
       </c>
-      <c r="AG40" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH40" s="8" t="s">
         <v>166</v>
       </c>
@@ -5008,10 +5171,13 @@
         <v>166</v>
       </c>
       <c r="AL40" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM40" s="8" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="41" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:39" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
         <v>280</v>
       </c>
@@ -5029,80 +5195,78 @@
         <v>157</v>
       </c>
       <c r="G41" s="8"/>
-      <c r="H41" s="8">
+      <c r="H41" s="8"/>
+      <c r="I41" s="8">
         <v>1319047328</v>
       </c>
-      <c r="I41" s="8">
+      <c r="J41" s="8">
         <v>1410284216</v>
       </c>
-      <c r="J41" s="8" t="s">
+      <c r="K41" s="8" t="s">
         <v>235</v>
       </c>
-      <c r="K41" s="8">
+      <c r="L41" s="8">
         <v>10000</v>
       </c>
-      <c r="L41" s="8"/>
-      <c r="M41" s="14">
+      <c r="M41" s="8"/>
+      <c r="N41" s="14">
         <v>46153</v>
       </c>
-      <c r="N41" s="14"/>
-      <c r="O41" s="8" t="s">
+      <c r="O41" s="14"/>
+      <c r="P41" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="P41" s="14">
+      <c r="Q41" s="14">
         <v>36835</v>
       </c>
-      <c r="Q41" s="15">
+      <c r="R41" s="15">
         <v>5579571190</v>
       </c>
-      <c r="R41" s="8" t="s">
+      <c r="S41" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="S41" s="15">
+      <c r="T41" s="15">
         <v>1731580505955</v>
       </c>
-      <c r="T41" s="8" t="s">
+      <c r="U41" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="U41" s="8" t="s">
+      <c r="V41" s="8" t="s">
         <v>216</v>
       </c>
-      <c r="V41" s="8" t="s">
+      <c r="W41" s="8" t="s">
         <v>236</v>
       </c>
-      <c r="W41" s="8" t="s">
+      <c r="X41" s="8" t="s">
         <v>237</v>
       </c>
-      <c r="X41" s="8">
+      <c r="Y41" s="8">
         <v>1834674262</v>
       </c>
-      <c r="Y41" s="8" t="s">
+      <c r="Z41" s="8" t="s">
         <v>238</v>
       </c>
-      <c r="Z41" s="8" t="s">
+      <c r="AA41" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="AA41" s="8" t="s">
+      <c r="AB41" s="8" t="s">
         <v>239</v>
       </c>
-      <c r="AB41" s="8" t="s">
+      <c r="AC41" s="8" t="s">
         <v>162</v>
-      </c>
-      <c r="AC41" s="8" t="s">
-        <v>241</v>
       </c>
       <c r="AD41" s="8" t="s">
         <v>241</v>
       </c>
       <c r="AE41" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="AF41" s="8" t="s">
         <v>237</v>
       </c>
-      <c r="AF41" s="8" t="s">
+      <c r="AG41" s="8" t="s">
         <v>240</v>
       </c>
-      <c r="AG41" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH41" s="8" t="s">
         <v>166</v>
       </c>
@@ -5116,10 +5280,13 @@
         <v>166</v>
       </c>
       <c r="AL41" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM41" s="8" t="s">
         <v>359</v>
       </c>
     </row>
-    <row r="42" spans="1:38" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:39" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="8" t="s">
         <v>280</v>
       </c>
@@ -5139,68 +5306,66 @@
         <v>284</v>
       </c>
       <c r="G42" s="8"/>
-      <c r="H42" s="8">
-        <v>1918580928</v>
-      </c>
+      <c r="H42" s="8"/>
       <c r="I42" s="8">
         <v>1918580928</v>
       </c>
-      <c r="J42" s="8"/>
+      <c r="J42" s="8">
+        <v>1918580928</v>
+      </c>
       <c r="K42" s="8"/>
       <c r="L42" s="8"/>
-      <c r="M42" s="14">
+      <c r="M42" s="8"/>
+      <c r="N42" s="14">
         <v>45972</v>
       </c>
-      <c r="N42" s="14"/>
-      <c r="O42" s="8" t="s">
+      <c r="O42" s="14"/>
+      <c r="P42" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="P42" s="14">
+      <c r="Q42" s="14">
         <v>30051</v>
       </c>
-      <c r="Q42" s="15">
+      <c r="R42" s="15">
         <v>4813347974417</v>
       </c>
-      <c r="R42" s="8" t="s">
+      <c r="S42" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="S42" s="15">
+      <c r="T42" s="15">
         <v>7017017975193</v>
       </c>
-      <c r="T42" s="8"/>
       <c r="U42" s="8"/>
       <c r="V42" s="8"/>
-      <c r="W42" s="8" t="s">
+      <c r="W42" s="8"/>
+      <c r="X42" s="8" t="s">
         <v>288</v>
       </c>
-      <c r="X42" s="8">
+      <c r="Y42" s="8">
         <v>1712436301</v>
       </c>
-      <c r="Y42" s="8" t="s">
+      <c r="Z42" s="8" t="s">
         <v>161</v>
       </c>
-      <c r="Z42" s="8" t="s">
+      <c r="AA42" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="AA42" s="8"/>
-      <c r="AB42" s="8" t="s">
+      <c r="AB42" s="8"/>
+      <c r="AC42" s="8" t="s">
         <v>173</v>
-      </c>
-      <c r="AC42" s="8" t="s">
-        <v>287</v>
       </c>
       <c r="AD42" s="8" t="s">
         <v>287</v>
       </c>
       <c r="AE42" s="8" t="s">
+        <v>287</v>
+      </c>
+      <c r="AF42" s="8" t="s">
         <v>285</v>
       </c>
-      <c r="AF42" s="8" t="s">
+      <c r="AG42" s="8" t="s">
         <v>286</v>
       </c>
-      <c r="AG42" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH42" s="8" t="s">
         <v>166</v>
       </c>
@@ -5214,10 +5379,13 @@
         <v>166</v>
       </c>
       <c r="AL42" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM42" s="8" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="43" spans="1:38" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:39" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="8" t="s">
         <v>280</v>
       </c>
@@ -5233,74 +5401,71 @@
       <c r="F43" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="H43" s="8">
+      <c r="I43" s="8">
         <v>1737576537</v>
       </c>
-      <c r="I43" s="8">
+      <c r="J43" s="8">
         <v>1410589082</v>
       </c>
-      <c r="J43" s="8" t="s">
+      <c r="K43" s="8" t="s">
         <v>303</v>
       </c>
-      <c r="K43" s="8">
+      <c r="L43" s="8">
         <v>10000</v>
       </c>
-      <c r="M43" s="14">
+      <c r="N43" s="14">
         <v>46174</v>
       </c>
-      <c r="N43" s="14"/>
-      <c r="O43" s="8" t="s">
+      <c r="O43" s="14"/>
+      <c r="P43" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="P43" s="14">
+      <c r="Q43" s="14">
         <v>32203</v>
       </c>
-      <c r="Q43" s="15">
+      <c r="R43" s="15">
         <v>1947866297</v>
       </c>
-      <c r="R43" s="8" t="s">
+      <c r="S43" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="S43" s="15"/>
-      <c r="T43" s="8" t="s">
+      <c r="T43" s="15"/>
+      <c r="U43" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="V43" s="8" t="s">
+      <c r="W43" s="8" t="s">
         <v>304</v>
       </c>
-      <c r="W43" s="8" t="s">
+      <c r="X43" s="8" t="s">
         <v>305</v>
       </c>
-      <c r="X43" s="8">
+      <c r="Y43" s="8">
         <v>1338582931</v>
       </c>
-      <c r="Y43" s="8" t="s">
+      <c r="Z43" s="8" t="s">
         <v>209</v>
       </c>
-      <c r="Z43" s="8" t="s">
+      <c r="AA43" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="AA43" s="8" t="s">
+      <c r="AB43" s="8" t="s">
         <v>239</v>
       </c>
-      <c r="AB43" s="8" t="s">
+      <c r="AC43" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="AC43" s="8" t="s">
+      <c r="AD43" s="8" t="s">
         <v>307</v>
       </c>
-      <c r="AD43" s="8" t="s">
+      <c r="AE43" s="8" t="s">
         <v>306</v>
       </c>
-      <c r="AE43" s="8" t="s">
+      <c r="AF43" s="8" t="s">
         <v>308</v>
       </c>
-      <c r="AF43" s="8" t="s">
+      <c r="AG43" s="8" t="s">
         <v>309</v>
       </c>
-      <c r="AG43" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH43" s="8" t="s">
         <v>166</v>
       </c>
@@ -5314,10 +5479,13 @@
         <v>166</v>
       </c>
       <c r="AL43" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM43" s="8" t="s">
         <v>359</v>
       </c>
     </row>
-    <row r="44" spans="1:38" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:39" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="9" t="s">
         <v>278</v>
       </c>
@@ -5333,29 +5501,26 @@
       <c r="F44" s="8" t="s">
         <v>284</v>
       </c>
-      <c r="H44" s="8">
+      <c r="I44" s="8">
         <v>1911229913</v>
       </c>
-      <c r="I44" s="8">
+      <c r="J44" s="8">
         <v>1923909896</v>
       </c>
-      <c r="M44" s="14">
+      <c r="N44" s="14">
         <v>43709</v>
       </c>
-      <c r="N44" s="14"/>
-      <c r="O44" s="8" t="s">
+      <c r="O44" s="14"/>
+      <c r="P44" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="P44" s="14">
+      <c r="Q44" s="14">
         <v>29571</v>
       </c>
-      <c r="Q44" s="15">
+      <c r="R44" s="15">
         <v>4201594605</v>
       </c>
-      <c r="S44" s="15"/>
-      <c r="AG44" s="8" t="s">
-        <v>166</v>
-      </c>
+      <c r="T44" s="15"/>
       <c r="AH44" s="8" t="s">
         <v>166</v>
       </c>
@@ -5369,10 +5534,13 @@
         <v>166</v>
       </c>
       <c r="AL44" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM44" s="8" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="45" spans="1:38" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:39" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="9" t="s">
         <v>278</v>
       </c>
@@ -5388,29 +5556,26 @@
       <c r="F45" s="8" t="s">
         <v>284</v>
       </c>
-      <c r="H45" s="8">
-        <v>1911266077</v>
-      </c>
       <c r="I45" s="8">
         <v>1911266077</v>
       </c>
-      <c r="M45" s="14">
+      <c r="J45" s="8">
+        <v>1911266077</v>
+      </c>
+      <c r="N45" s="14">
         <v>44378</v>
       </c>
-      <c r="N45" s="14"/>
-      <c r="O45" s="8" t="s">
+      <c r="O45" s="14"/>
+      <c r="P45" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="P45" s="14">
+      <c r="Q45" s="14">
         <v>35495</v>
       </c>
-      <c r="Q45" s="15">
+      <c r="R45" s="15">
         <v>1.9974815471E+16</v>
       </c>
-      <c r="S45" s="15"/>
-      <c r="AG45" s="8" t="s">
-        <v>166</v>
-      </c>
+      <c r="T45" s="15"/>
       <c r="AH45" s="8" t="s">
         <v>166</v>
       </c>
@@ -5424,10 +5589,13 @@
         <v>166</v>
       </c>
       <c r="AL45" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM45" s="8" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="46" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A46" s="8" t="s">
         <v>280</v>
       </c>
@@ -5443,78 +5611,76 @@
       <c r="F46" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="H46" s="5">
+      <c r="G46" s="8"/>
+      <c r="I46" s="5">
         <v>1921437014</v>
       </c>
-      <c r="I46" s="5">
+      <c r="J46" s="5">
         <v>1410167293</v>
       </c>
-      <c r="J46" s="5" t="s">
+      <c r="K46" s="5" t="s">
         <v>350</v>
       </c>
-      <c r="K46" s="8">
+      <c r="L46" s="8">
         <v>10000</v>
       </c>
-      <c r="M46" s="6">
+      <c r="N46" s="6">
         <v>46174</v>
       </c>
-      <c r="O46" s="8" t="s">
+      <c r="P46" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="P46" s="6">
+      <c r="Q46" s="6">
         <v>35929</v>
       </c>
-      <c r="Q46" s="7">
+      <c r="R46" s="7">
         <v>5112217939</v>
       </c>
-      <c r="R46" s="8" t="s">
+      <c r="S46" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="S46" s="7">
+      <c r="T46" s="7">
         <v>1731570644612</v>
       </c>
-      <c r="T46" s="8" t="s">
+      <c r="U46" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="U46" s="8" t="s">
+      <c r="V46" s="8" t="s">
         <v>216</v>
       </c>
-      <c r="V46" s="5" t="s">
+      <c r="W46" s="5" t="s">
         <v>351</v>
       </c>
-      <c r="W46" s="5" t="s">
+      <c r="X46" s="5" t="s">
         <v>361</v>
       </c>
-      <c r="X46" s="5">
+      <c r="Y46" s="5">
         <v>1946653418</v>
       </c>
-      <c r="Y46" s="5" t="s">
+      <c r="Z46" s="5" t="s">
         <v>238</v>
       </c>
-      <c r="Z46" s="5" t="s">
+      <c r="AA46" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="AA46" s="5" t="s">
+      <c r="AB46" s="5" t="s">
         <v>362</v>
       </c>
-      <c r="AB46" s="8" t="s">
+      <c r="AC46" s="8" t="s">
         <v>148</v>
-      </c>
-      <c r="AC46" s="5" t="s">
-        <v>363</v>
       </c>
       <c r="AD46" s="5" t="s">
         <v>363</v>
       </c>
       <c r="AE46" s="5" t="s">
+        <v>363</v>
+      </c>
+      <c r="AF46" s="5" t="s">
         <v>361</v>
       </c>
-      <c r="AF46" s="5" t="s">
+      <c r="AG46" s="5" t="s">
         <v>364</v>
       </c>
-      <c r="AG46" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH46" s="8" t="s">
         <v>166</v>
       </c>
@@ -5528,10 +5694,13 @@
         <v>166</v>
       </c>
       <c r="AL46" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM46" s="8" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="47" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A47" s="8" t="s">
         <v>280</v>
       </c>
@@ -5547,66 +5716,64 @@
       <c r="F47" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="H47" s="5">
+      <c r="G47" s="8"/>
+      <c r="I47" s="5">
         <v>1605632547</v>
       </c>
-      <c r="I47" s="5">
+      <c r="J47" s="5">
         <v>1410449332</v>
       </c>
-      <c r="J47" s="5" t="s">
+      <c r="K47" s="5" t="s">
         <v>368</v>
       </c>
-      <c r="K47" s="8">
+      <c r="L47" s="8">
         <v>10000</v>
       </c>
-      <c r="M47" s="6">
+      <c r="N47" s="6">
         <v>46174</v>
       </c>
-      <c r="O47" s="8" t="s">
+      <c r="P47" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="P47" s="6">
+      <c r="Q47" s="6">
         <v>38475</v>
       </c>
-      <c r="Q47" s="7">
+      <c r="R47" s="7">
         <v>9587105819</v>
       </c>
-      <c r="V47" s="5" t="s">
+      <c r="W47" s="5" t="s">
         <v>369</v>
       </c>
-      <c r="W47" s="5" t="s">
+      <c r="X47" s="5" t="s">
         <v>370</v>
       </c>
-      <c r="X47" s="5">
+      <c r="Y47" s="5">
         <v>1913711156</v>
       </c>
-      <c r="Y47" s="5" t="s">
+      <c r="Z47" s="5" t="s">
         <v>238</v>
       </c>
-      <c r="Z47" s="5" t="s">
+      <c r="AA47" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="AA47" s="5" t="s">
+      <c r="AB47" s="5" t="s">
         <v>371</v>
       </c>
-      <c r="AB47" s="8" t="s">
+      <c r="AC47" s="8" t="s">
         <v>162</v>
-      </c>
-      <c r="AC47" s="5" t="s">
-        <v>372</v>
       </c>
       <c r="AD47" s="5" t="s">
         <v>372</v>
       </c>
       <c r="AE47" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="AF47" s="5" t="s">
         <v>370</v>
       </c>
-      <c r="AF47" s="5" t="s">
+      <c r="AG47" s="5" t="s">
         <v>373</v>
       </c>
-      <c r="AG47" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH47" s="8" t="s">
         <v>166</v>
       </c>
@@ -5620,10 +5787,13 @@
         <v>166</v>
       </c>
       <c r="AL47" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM47" s="8" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="48" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A48" s="9" t="s">
         <v>278</v>
       </c>
@@ -5636,63 +5806,60 @@
       <c r="F48" s="5" t="s">
         <v>271</v>
       </c>
-      <c r="H48" s="5">
+      <c r="I48" s="5">
         <v>1966727374</v>
       </c>
-      <c r="I48" s="9">
+      <c r="J48" s="9">
         <v>1935597976</v>
       </c>
-      <c r="J48" s="5" t="s">
+      <c r="K48" s="5" t="s">
         <v>388</v>
       </c>
-      <c r="M48" s="6">
+      <c r="N48" s="6">
         <v>46204</v>
       </c>
-      <c r="O48" s="8" t="s">
+      <c r="P48" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="P48" s="6">
+      <c r="Q48" s="6">
         <v>28705</v>
       </c>
-      <c r="Q48" s="7">
+      <c r="R48" s="7">
         <v>2400568289</v>
       </c>
-      <c r="V48" s="5" t="s">
+      <c r="W48" s="5" t="s">
         <v>379</v>
       </c>
-      <c r="W48" s="5" t="s">
+      <c r="X48" s="5" t="s">
         <v>380</v>
       </c>
-      <c r="X48" s="5">
+      <c r="Y48" s="5">
         <v>1937936060</v>
       </c>
-      <c r="Y48" s="5" t="s">
+      <c r="Z48" s="5" t="s">
         <v>209</v>
       </c>
-      <c r="Z48" s="5" t="s">
+      <c r="AA48" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="AA48" s="8" t="s">
+      <c r="AB48" s="8" t="s">
         <v>239</v>
       </c>
-      <c r="AB48" s="5" t="s">
+      <c r="AC48" s="5" t="s">
         <v>381</v>
-      </c>
-      <c r="AC48" s="5" t="s">
-        <v>382</v>
       </c>
       <c r="AD48" s="5" t="s">
         <v>382</v>
       </c>
       <c r="AE48" s="5" t="s">
+        <v>382</v>
+      </c>
+      <c r="AF48" s="5" t="s">
         <v>383</v>
       </c>
-      <c r="AF48" s="5" t="s">
+      <c r="AG48" s="5" t="s">
         <v>384</v>
       </c>
-      <c r="AG48" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH48" s="8" t="s">
         <v>166</v>
       </c>
@@ -5706,10 +5873,13 @@
         <v>166</v>
       </c>
       <c r="AL48" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM48" s="8" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="49" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A49" s="8" t="s">
         <v>280</v>
       </c>
@@ -5722,63 +5892,61 @@
       <c r="F49" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="H49" s="5">
-        <v>1410490086</v>
-      </c>
+      <c r="G49" s="8"/>
       <c r="I49" s="5">
         <v>1410490086</v>
       </c>
-      <c r="J49" s="5" t="s">
+      <c r="J49" s="5">
+        <v>1410490086</v>
+      </c>
+      <c r="K49" s="5" t="s">
         <v>387</v>
       </c>
-      <c r="M49" s="6">
+      <c r="N49" s="6">
         <v>46204</v>
       </c>
-      <c r="O49" s="8" t="s">
+      <c r="P49" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="P49" s="6">
+      <c r="Q49" s="6">
         <v>32854</v>
       </c>
-      <c r="Q49" s="7">
+      <c r="R49" s="7">
         <v>4813386925537</v>
       </c>
-      <c r="V49" s="5" t="s">
+      <c r="W49" s="5" t="s">
         <v>389</v>
       </c>
-      <c r="W49" s="5" t="s">
+      <c r="X49" s="5" t="s">
         <v>390</v>
       </c>
-      <c r="X49" s="5">
+      <c r="Y49" s="5">
         <v>1796245290</v>
       </c>
-      <c r="Y49" s="5" t="s">
+      <c r="Z49" s="5" t="s">
         <v>391</v>
       </c>
-      <c r="Z49" s="5" t="s">
+      <c r="AA49" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="AA49" s="5" t="s">
+      <c r="AB49" s="5" t="s">
         <v>392</v>
       </c>
-      <c r="AB49" s="8" t="s">
+      <c r="AC49" s="8" t="s">
         <v>162</v>
-      </c>
-      <c r="AC49" s="5" t="s">
-        <v>393</v>
       </c>
       <c r="AD49" s="5" t="s">
         <v>393</v>
       </c>
       <c r="AE49" s="5" t="s">
+        <v>393</v>
+      </c>
+      <c r="AF49" s="5" t="s">
         <v>394</v>
       </c>
-      <c r="AF49" s="5" t="s">
+      <c r="AG49" s="5" t="s">
         <v>395</v>
       </c>
-      <c r="AG49" s="8" t="s">
-        <v>166</v>
-      </c>
       <c r="AH49" s="8" t="s">
         <v>166</v>
       </c>
@@ -5792,13 +5960,16 @@
         <v>166</v>
       </c>
       <c r="AL49" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM49" s="8" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="50" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:39" x14ac:dyDescent="0.25">
       <c r="E50" s="8"/>
     </row>
-    <row r="51" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:39" x14ac:dyDescent="0.25">
       <c r="E51" s="8"/>
     </row>
   </sheetData>
@@ -5806,10 +5977,10 @@
   <conditionalFormatting sqref="C1:C1048576">
     <cfRule type="duplicateValues" dxfId="2" priority="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J1:J1048576">
+  <conditionalFormatting sqref="K1:K1048576">
     <cfRule type="duplicateValues" dxfId="1" priority="4"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q1:Q1048576">
+  <conditionalFormatting sqref="R1:R1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="3"/>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: enhance employee management with new employee types and UI updates fix: improve data handling in GA live report and resync script
</commit_message>
<xml_diff>
--- a/backend/data/emplyoees.xlsx
+++ b/backend/data/emplyoees.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\emil\projects\Orange-Flow-Next-Js\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81868FA2-C0E0-4C32-9D0D-42A67BCCF058}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{253A4515-038B-4F08-87B7-3233D2F9C924}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AM$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AM$50</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="955" uniqueCount="423">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="980" uniqueCount="434">
   <si>
     <t>DMS_CODE</t>
   </si>
@@ -1308,6 +1308,39 @@
   </si>
   <si>
     <t>SR-13</t>
+  </si>
+  <si>
+    <t>Kishoreganj</t>
+  </si>
+  <si>
+    <t>masummia</t>
+  </si>
+  <si>
+    <t>MER-MYMVAI0222</t>
+  </si>
+  <si>
+    <t>Masum Mia</t>
+  </si>
+  <si>
+    <t>R591269</t>
+  </si>
+  <si>
+    <t>Mithamoin</t>
+  </si>
+  <si>
+    <t>Yeasin</t>
+  </si>
+  <si>
+    <t>Muktijoddha Abdul Haque Govt. College</t>
+  </si>
+  <si>
+    <t>Nobabpur, Mithamoin, Kishoreganj</t>
+  </si>
+  <si>
+    <t>Sojol Mia</t>
+  </si>
+  <si>
+    <t>Khairunnesa</t>
   </si>
 </sst>
 </file>
@@ -4365,6 +4398,9 @@
       <c r="F33" s="8" t="s">
         <v>157</v>
       </c>
+      <c r="H33" s="8">
+        <v>1410678746</v>
+      </c>
       <c r="I33" s="8">
         <v>1786080093</v>
       </c>
@@ -4462,7 +4498,9 @@
         <v>157</v>
       </c>
       <c r="G34" s="8"/>
-      <c r="H34" s="8"/>
+      <c r="H34" s="8">
+        <v>1410071973</v>
+      </c>
       <c r="I34" s="8">
         <v>1410071973</v>
       </c>
@@ -4567,7 +4605,9 @@
         <v>157</v>
       </c>
       <c r="G35" s="8"/>
-      <c r="H35" s="8"/>
+      <c r="H35" s="8">
+        <v>1410240211</v>
+      </c>
       <c r="I35" s="8">
         <v>1410240211</v>
       </c>
@@ -4670,7 +4710,9 @@
         <v>157</v>
       </c>
       <c r="G36" s="8"/>
-      <c r="H36" s="8"/>
+      <c r="H36" s="8">
+        <v>1410436602</v>
+      </c>
       <c r="I36" s="8">
         <v>1917787990</v>
       </c>
@@ -4773,7 +4815,9 @@
         <v>157</v>
       </c>
       <c r="G37" s="8"/>
-      <c r="H37" s="8"/>
+      <c r="H37" s="8">
+        <v>1410213723</v>
+      </c>
       <c r="I37" s="8">
         <v>1305213723</v>
       </c>
@@ -4876,7 +4920,9 @@
         <v>157</v>
       </c>
       <c r="G38" s="8"/>
-      <c r="H38" s="8"/>
+      <c r="H38" s="8">
+        <v>1410173774</v>
+      </c>
       <c r="I38" s="8">
         <v>1990757830</v>
       </c>
@@ -4977,7 +5023,9 @@
         <v>157</v>
       </c>
       <c r="G39" s="8"/>
-      <c r="H39" s="8"/>
+      <c r="H39" s="8">
+        <v>1410720313</v>
+      </c>
       <c r="I39" s="8">
         <v>1763122889</v>
       </c>
@@ -5086,7 +5134,9 @@
         <v>157</v>
       </c>
       <c r="G40" s="8"/>
-      <c r="H40" s="8"/>
+      <c r="H40" s="8">
+        <v>1410031485</v>
+      </c>
       <c r="I40" s="8">
         <v>1984397910</v>
       </c>
@@ -5195,7 +5245,9 @@
         <v>157</v>
       </c>
       <c r="G41" s="8"/>
-      <c r="H41" s="8"/>
+      <c r="H41" s="8">
+        <v>1410284216</v>
+      </c>
       <c r="I41" s="8">
         <v>1319047328</v>
       </c>
@@ -5306,7 +5358,9 @@
         <v>284</v>
       </c>
       <c r="G42" s="8"/>
-      <c r="H42" s="8"/>
+      <c r="H42" s="8">
+        <v>1918580928</v>
+      </c>
       <c r="I42" s="8">
         <v>1918580928</v>
       </c>
@@ -5401,6 +5455,9 @@
       <c r="F43" s="8" t="s">
         <v>157</v>
       </c>
+      <c r="H43" s="8">
+        <v>1410589082</v>
+      </c>
       <c r="I43" s="8">
         <v>1737576537</v>
       </c>
@@ -5612,6 +5669,9 @@
         <v>157</v>
       </c>
       <c r="G46" s="8"/>
+      <c r="H46" s="5">
+        <v>1410167293</v>
+      </c>
       <c r="I46" s="5">
         <v>1921437014</v>
       </c>
@@ -5717,6 +5777,9 @@
         <v>157</v>
       </c>
       <c r="G47" s="8"/>
+      <c r="H47" s="5">
+        <v>1410449332</v>
+      </c>
       <c r="I47" s="5">
         <v>1605632547</v>
       </c>
@@ -5893,6 +5956,9 @@
         <v>157</v>
       </c>
       <c r="G49" s="8"/>
+      <c r="H49" s="5">
+        <v>1410490086</v>
+      </c>
       <c r="I49" s="5">
         <v>1410490086</v>
       </c>
@@ -5914,6 +5980,15 @@
       <c r="R49" s="7">
         <v>4813386925537</v>
       </c>
+      <c r="S49" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="T49" s="7">
+        <v>1877348858106</v>
+      </c>
+      <c r="U49" s="5" t="s">
+        <v>423</v>
+      </c>
       <c r="W49" s="5" t="s">
         <v>389</v>
       </c>
@@ -5967,7 +6042,93 @@
       </c>
     </row>
     <row r="50" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="E50" s="8"/>
+      <c r="A50" s="9" t="s">
+        <v>279</v>
+      </c>
+      <c r="B50" s="5" t="s">
+        <v>424</v>
+      </c>
+      <c r="C50" s="5" t="s">
+        <v>425</v>
+      </c>
+      <c r="E50" s="8" t="s">
+        <v>426</v>
+      </c>
+      <c r="F50" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="I50" s="5">
+        <v>1568659826</v>
+      </c>
+      <c r="J50" s="5">
+        <v>1999969026</v>
+      </c>
+      <c r="K50" s="5" t="s">
+        <v>427</v>
+      </c>
+      <c r="N50" s="6">
+        <v>46204</v>
+      </c>
+      <c r="P50" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="Q50" s="6">
+        <v>38390</v>
+      </c>
+      <c r="R50" s="7">
+        <v>6028880471</v>
+      </c>
+      <c r="W50" s="5" t="s">
+        <v>428</v>
+      </c>
+      <c r="X50" s="5" t="s">
+        <v>429</v>
+      </c>
+      <c r="Y50" s="5">
+        <v>1824099740</v>
+      </c>
+      <c r="Z50" s="5" t="s">
+        <v>391</v>
+      </c>
+      <c r="AA50" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="AB50" s="5" t="s">
+        <v>430</v>
+      </c>
+      <c r="AC50" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="AD50" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="AE50" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="AF50" s="5" t="s">
+        <v>432</v>
+      </c>
+      <c r="AG50" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="AH50" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="AI50" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="AJ50" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="AK50" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="AL50" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM50" s="8" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="51" spans="1:39" x14ac:dyDescent="0.25">
       <c r="E51" s="8"/>

</xml_diff>

<commit_message>
feat: update wait_for_selector to use 'attached' state for improved reliability in SIM tasks
</commit_message>
<xml_diff>
--- a/backend/data/emplyoees.xlsx
+++ b/backend/data/emplyoees.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\emil\projects\Orange-Flow-Next-Js\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{253A4515-038B-4F08-87B7-3233D2F9C924}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9CAF51F-A8E4-4B01-8A24-623D82A0643E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -5770,7 +5770,7 @@
       <c r="C47" s="5" t="s">
         <v>366</v>
       </c>
-      <c r="E47" s="8" t="s">
+      <c r="E47" s="18" t="s">
         <v>360</v>
       </c>
       <c r="F47" s="8" t="s">
@@ -5853,7 +5853,7 @@
         <v>166</v>
       </c>
       <c r="AM47" s="8" t="s">
-        <v>74</v>
+        <v>359</v>
       </c>
     </row>
     <row r="48" spans="1:39" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
feat: add stock management components and functionality
- Introduced ModeToggle component for switching between house and employee stock modes.
- Created StockEntryModal for adding and editing stock entries, including employee and product selection.
- Implemented SubcategoryModal to display subcategory details for selected categories.
- Added TransferModal for transferring stock between employees and houses.
- Developed custom hooks useMyShift and useShifts for managing shift data.
- Defined new types for sales and shifts to support the new features.
- Updated navigation to include Sales & Stock section.
- Established stock-related types for better type safety and clarity in the codebase.
</commit_message>
<xml_diff>
--- a/backend/data/emplyoees.xlsx
+++ b/backend/data/emplyoees.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\emil\projects\Orange-Flow-Next-Js\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9CAF51F-A8E4-4B01-8A24-623D82A0643E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E512602-9657-4539-9676-9EEFA55FFB1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="980" uniqueCount="434">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="983" uniqueCount="434">
   <si>
     <t>DMS_CODE</t>
   </si>
@@ -5890,6 +5890,18 @@
       <c r="R48" s="7">
         <v>2400568289</v>
       </c>
+      <c r="S48" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="T48" s="7">
+        <v>1731580521769</v>
+      </c>
+      <c r="U48" s="8" t="s">
+        <v>171</v>
+      </c>
+      <c r="V48" s="8" t="s">
+        <v>216</v>
+      </c>
       <c r="W48" s="5" t="s">
         <v>379</v>
       </c>

</xml_diff>

<commit_message>
feat: optimize serial number batch creation and enhance error handling in sync process
</commit_message>
<xml_diff>
--- a/backend/data/emplyoees.xlsx
+++ b/backend/data/emplyoees.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\emil\projects\Orange-Flow-Next-Js\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E512602-9657-4539-9676-9EEFA55FFB1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DB94E96-5991-43DB-B307-1335D2DEEE0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1469,7 +1469,15 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -5016,7 +5024,7 @@
         <v>213</v>
       </c>
       <c r="D39" s="8"/>
-      <c r="E39" s="8" t="s">
+      <c r="E39" s="18" t="s">
         <v>214</v>
       </c>
       <c r="F39" s="8" t="s">
@@ -5113,7 +5121,7 @@
         <v>166</v>
       </c>
       <c r="AM39" s="8" t="s">
-        <v>74</v>
+        <v>359</v>
       </c>
     </row>
     <row r="40" spans="1:39" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -6148,13 +6156,13 @@
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K1:K1048576">
-    <cfRule type="duplicateValues" dxfId="1" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="R1:R1048576">
-    <cfRule type="duplicateValues" dxfId="0" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="3"/>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
feat: add bulk stock item creation functionality and update related schemas
</commit_message>
<xml_diff>
--- a/backend/data/emplyoees.xlsx
+++ b/backend/data/emplyoees.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\emil\projects\Orange-Flow-Next-Js\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DB94E96-5991-43DB-B307-1335D2DEEE0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05B45384-1B9C-4186-9C45-55B103DD6CB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="983" uniqueCount="434">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1004" uniqueCount="439">
   <si>
     <t>DMS_CODE</t>
   </si>
@@ -1341,6 +1341,21 @@
   </si>
   <si>
     <t>Khairunnesa</t>
+  </si>
+  <si>
+    <t>Fahim Hossin</t>
+  </si>
+  <si>
+    <t>Monir</t>
+  </si>
+  <si>
+    <t>Hazi Asmot College</t>
+  </si>
+  <si>
+    <t>Monir Hossen</t>
+  </si>
+  <si>
+    <t>Suma Begum</t>
   </si>
 </sst>
 </file>
@@ -1469,15 +1484,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="3">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -6151,18 +6158,98 @@
       </c>
     </row>
     <row r="51" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="E51" s="8"/>
+      <c r="A51" s="8" t="s">
+        <v>280</v>
+      </c>
+      <c r="E51" s="8" t="s">
+        <v>434</v>
+      </c>
+      <c r="F51" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="I51" s="5">
+        <v>1733466898</v>
+      </c>
+      <c r="L51" s="5">
+        <v>10000</v>
+      </c>
+      <c r="N51" s="6">
+        <v>46235</v>
+      </c>
+      <c r="P51" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="Q51" s="6">
+        <v>37491</v>
+      </c>
+      <c r="R51" s="7">
+        <v>8713578253</v>
+      </c>
+      <c r="U51" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="W51" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="X51" s="5" t="s">
+        <v>435</v>
+      </c>
+      <c r="Y51" s="5">
+        <v>1341114046</v>
+      </c>
+      <c r="Z51" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="AA51" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="AB51" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="AC51" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="AD51" s="5" t="s">
+        <v>382</v>
+      </c>
+      <c r="AE51" s="5" t="s">
+        <v>382</v>
+      </c>
+      <c r="AF51" s="5" t="s">
+        <v>437</v>
+      </c>
+      <c r="AG51" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="AH51" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="AI51" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="AJ51" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="AK51" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="AL51" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM51" s="8" t="s">
+        <v>74</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K1:K1048576">
-    <cfRule type="duplicateValues" dxfId="2" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="R1:R1048576">
-    <cfRule type="duplicateValues" dxfId="1" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="3"/>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
feat(stock): enhance transfer functionality with multiple product lines and improved UI
- Updated ModalShell to accept a 'wide' prop for better layout control.
- Refactored transfer form to support multiple product lines, allowing users to add, update, and remove transfer lines dynamically.
- Adjusted validation to ensure proper quantity checks against available stock for each product line.
- Modified API request to handle bulk transfers of multiple products.
- Updated translations for improved clarity and consistency in the UI.
</commit_message>
<xml_diff>
--- a/backend/data/emplyoees.xlsx
+++ b/backend/data/emplyoees.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\emil\projects\Orange-Flow-Next-Js\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05B45384-1B9C-4186-9C45-55B103DD6CB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6B356D5-22F3-4DC2-960F-73AA0E908A22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1004" uniqueCount="439">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1006" uniqueCount="441">
   <si>
     <t>DMS_CODE</t>
   </si>
@@ -1356,6 +1356,12 @@
   </si>
   <si>
     <t>Suma Begum</t>
+  </si>
+  <si>
+    <t>MER-RYZBRB0133</t>
+  </si>
+  <si>
+    <t>R649191</t>
   </si>
 </sst>
 </file>
@@ -6161,14 +6167,26 @@
       <c r="A51" s="8" t="s">
         <v>280</v>
       </c>
+      <c r="C51" s="5" t="s">
+        <v>439</v>
+      </c>
       <c r="E51" s="8" t="s">
         <v>434</v>
       </c>
       <c r="F51" s="8" t="s">
         <v>157</v>
       </c>
+      <c r="H51" s="5">
+        <v>1410760970</v>
+      </c>
       <c r="I51" s="5">
         <v>1733466898</v>
+      </c>
+      <c r="J51" s="5">
+        <v>1410760970</v>
+      </c>
+      <c r="K51" s="5" t="s">
+        <v>440</v>
       </c>
       <c r="L51" s="5">
         <v>10000</v>

</xml_diff>

<commit_message>
feat: enhance retailer ID retrieval for employees and include resigned RSOs in reports
</commit_message>
<xml_diff>
--- a/backend/data/emplyoees.xlsx
+++ b/backend/data/emplyoees.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\emil\projects\Orange-Flow-Next-Js\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6B356D5-22F3-4DC2-960F-73AA0E908A22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21A9BCFC-9C9B-48C5-AF59-B4D67A9CF9D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="390" windowWidth="28800" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1006" uniqueCount="441">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1030" uniqueCount="446">
   <si>
     <t>DMS_CODE</t>
   </si>
@@ -1362,6 +1362,21 @@
   </si>
   <si>
     <t>R649191</t>
+  </si>
+  <si>
+    <t>Mahfuza Begum</t>
+  </si>
+  <si>
+    <t>Md. Saddam Hosan</t>
+  </si>
+  <si>
+    <t>RYZBRB01SUP02</t>
+  </si>
+  <si>
+    <t>Md. Hanif Mia</t>
+  </si>
+  <si>
+    <t>Shokhina Begum</t>
   </si>
 </sst>
 </file>
@@ -1825,7 +1840,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AM51"/>
+  <dimension ref="A1:AM52"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.5703125" style="5" bestFit="1" customWidth="1"/>
@@ -5372,7 +5387,7 @@
       <c r="D42" s="8" t="s">
         <v>282</v>
       </c>
-      <c r="E42" s="8" t="s">
+      <c r="E42" s="18" t="s">
         <v>283</v>
       </c>
       <c r="F42" s="8" t="s">
@@ -5457,7 +5472,7 @@
         <v>166</v>
       </c>
       <c r="AM42" s="8" t="s">
-        <v>74</v>
+        <v>359</v>
       </c>
     </row>
     <row r="43" spans="1:39" s="8" customFormat="1" x14ac:dyDescent="0.25">
@@ -6255,6 +6270,104 @@
         <v>166</v>
       </c>
       <c r="AM51" s="8" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="52" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A52" s="8" t="s">
+        <v>280</v>
+      </c>
+      <c r="C52" s="5" t="s">
+        <v>443</v>
+      </c>
+      <c r="E52" s="5" t="s">
+        <v>442</v>
+      </c>
+      <c r="F52" s="8" t="s">
+        <v>284</v>
+      </c>
+      <c r="H52" s="5">
+        <v>1410050892</v>
+      </c>
+      <c r="I52" s="5">
+        <v>1796672446</v>
+      </c>
+      <c r="J52" s="5">
+        <v>1410050892</v>
+      </c>
+      <c r="N52" s="6">
+        <v>46235</v>
+      </c>
+      <c r="P52" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="Q52" s="6">
+        <v>34587</v>
+      </c>
+      <c r="R52" s="7">
+        <v>6887047287</v>
+      </c>
+      <c r="S52" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="T52" s="7">
+        <v>1731010043834</v>
+      </c>
+      <c r="U52" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="V52" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="W52" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="X52" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="Y52" s="5">
+        <v>1792104219</v>
+      </c>
+      <c r="Z52" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="AA52" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="AB52" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="AC52" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="AD52" s="5" t="s">
+        <v>382</v>
+      </c>
+      <c r="AE52" s="5" t="s">
+        <v>382</v>
+      </c>
+      <c r="AF52" s="5" t="s">
+        <v>444</v>
+      </c>
+      <c r="AG52" s="5" t="s">
+        <v>445</v>
+      </c>
+      <c r="AH52" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="AI52" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="AJ52" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="AK52" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="AL52" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="AM52" s="8" t="s">
         <v>74</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: enhance recharge report with yesterday's C2C, C2S, and transaction count metrics
</commit_message>
<xml_diff>
--- a/backend/data/emplyoees.xlsx
+++ b/backend/data/emplyoees.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\emil\projects\Orange-Flow-Next-Js\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21A9BCFC-9C9B-48C5-AF59-B4D67A9CF9D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99CF7595-D50F-4620-BFBD-2FE3E7A076D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="390" windowWidth="28800" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="1170" windowWidth="28800" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -6185,7 +6185,7 @@
       <c r="C51" s="5" t="s">
         <v>439</v>
       </c>
-      <c r="E51" s="8" t="s">
+      <c r="E51" s="18" t="s">
         <v>434</v>
       </c>
       <c r="F51" s="8" t="s">
@@ -6270,7 +6270,7 @@
         <v>166</v>
       </c>
       <c r="AM51" s="8" t="s">
-        <v>74</v>
+        <v>359</v>
       </c>
     </row>
     <row r="52" spans="1:39" x14ac:dyDescent="0.25">

</xml_diff>